<commit_message>
Update LSP spreadsheet data
</commit_message>
<xml_diff>
--- a/data/20251229_LSP管理.xlsx
+++ b/data/20251229_LSP管理.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hiraizumitatsuya/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A91DD1F1-550F-48D5-B0C4-04028FE0273E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{09645455-26E2-4DFD-8999-22E8DD0D3AB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="33600" windowHeight="20500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2908" uniqueCount="394">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2896" uniqueCount="392">
   <si>
     <t>日付</t>
   </si>
@@ -1181,12 +1181,6 @@
   </si>
   <si>
     <t>JAL４８４</t>
-  </si>
-  <si>
-    <t>JAL153</t>
-  </si>
-  <si>
-    <t>三沢</t>
   </si>
   <si>
     <t>JAL113</t>
@@ -14700,8 +14694,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{3FCDC422-27B5-482E-BFE7-6645FF3F845A}" name="テーブル4" displayName="テーブル4" ref="A1:M265" totalsRowShown="0" headerRowDxfId="16" headerRowBorderDxfId="14" tableBorderDxfId="15" totalsRowBorderDxfId="13">
-  <autoFilter ref="A1:M265" xr:uid="{3FCDC422-27B5-482E-BFE7-6645FF3F845A}">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{3FCDC422-27B5-482E-BFE7-6645FF3F845A}" name="テーブル4" displayName="テーブル4" ref="A1:M263" totalsRowShown="0" headerRowDxfId="16" headerRowBorderDxfId="14" tableBorderDxfId="15" totalsRowBorderDxfId="13">
+  <autoFilter ref="A1:M263" xr:uid="{3FCDC422-27B5-482E-BFE7-6645FF3F845A}">
     <filterColumn colId="11">
       <filters blank="1"/>
     </filterColumn>
@@ -46445,7 +46439,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{82EF3C4E-F452-4BBC-81DB-9BE6F59D48AA}">
-  <dimension ref="A1:M319"/>
+  <dimension ref="A1:M317"/>
   <sheetFormatPr defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="4.28515625" bestFit="1" customWidth="1"/>
@@ -53810,12 +53804,12 @@
       </c>
       <c r="M216" s="15"/>
     </row>
-    <row r="217" spans="1:13">
+    <row r="217" spans="1:13" hidden="1">
       <c r="A217" s="14">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="B217" s="42">
-        <v>46177</v>
+        <v>46153</v>
       </c>
       <c r="C217" s="12" t="s">
         <v>293</v>
@@ -53827,19 +53821,21 @@
         <v>294</v>
       </c>
       <c r="F217" s="13">
-        <v>0.34375</v>
+        <v>0.44791666666666669</v>
       </c>
       <c r="G217" s="12" t="s">
-        <v>378</v>
+        <v>371</v>
       </c>
       <c r="H217" s="13">
-        <v>0.39583333333333331</v>
+        <v>0.49305555555555558</v>
       </c>
       <c r="I217" s="26"/>
       <c r="J217" s="15" t="s">
         <v>358</v>
       </c>
-      <c r="K217" s="22"/>
+      <c r="K217" s="22">
+        <v>0</v>
+      </c>
       <c r="L217" s="15" t="s">
         <v>297</v>
       </c>
@@ -53847,45 +53843,45 @@
     </row>
     <row r="218" spans="1:13">
       <c r="A218" s="14">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="B218" s="42">
-        <v>46177</v>
+        <v>46223</v>
       </c>
       <c r="C218" s="12" t="s">
         <v>293</v>
       </c>
       <c r="D218" s="12" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="E218" s="12" t="s">
-        <v>378</v>
+        <v>294</v>
       </c>
       <c r="F218" s="13">
-        <v>0.79861111111111116</v>
+        <v>0.2951388888888889</v>
       </c>
       <c r="G218" s="12" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="H218" s="13">
-        <v>0.85763888888888884</v>
+        <v>0.36458333333333331</v>
       </c>
       <c r="I218" s="26"/>
       <c r="J218" s="15" t="s">
         <v>358</v>
       </c>
-      <c r="K218" s="22"/>
-      <c r="L218" s="15" t="s">
-        <v>297</v>
-      </c>
+      <c r="K218" s="22">
+        <v>27740</v>
+      </c>
+      <c r="L218" s="15"/>
       <c r="M218" s="15"/>
     </row>
-    <row r="219" spans="1:13" hidden="1">
+    <row r="219" spans="1:13">
       <c r="A219" s="14">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="B219" s="42">
-        <v>46153</v>
+        <v>46229</v>
       </c>
       <c r="C219" s="12" t="s">
         <v>293</v>
@@ -53894,16 +53890,16 @@
         <v>379</v>
       </c>
       <c r="E219" s="12" t="s">
+        <v>295</v>
+      </c>
+      <c r="F219" s="13">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="G219" s="12" t="s">
         <v>294</v>
       </c>
-      <c r="F219" s="13">
-        <v>0.44791666666666669</v>
-      </c>
-      <c r="G219" s="12" t="s">
-        <v>371</v>
-      </c>
       <c r="H219" s="13">
-        <v>0.49305555555555558</v>
+        <v>0.48958333333333331</v>
       </c>
       <c r="I219" s="26"/>
       <c r="J219" s="15" t="s">
@@ -53912,17 +53908,15 @@
       <c r="K219" s="22">
         <v>0</v>
       </c>
-      <c r="L219" s="15" t="s">
-        <v>297</v>
-      </c>
+      <c r="L219" s="15"/>
       <c r="M219" s="15"/>
     </row>
     <row r="220" spans="1:13">
       <c r="A220" s="14">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="B220" s="42">
-        <v>46223</v>
+        <v>46182</v>
       </c>
       <c r="C220" s="12" t="s">
         <v>293</v>
@@ -53934,48 +53928,48 @@
         <v>294</v>
       </c>
       <c r="F220" s="13">
-        <v>0.2951388888888889</v>
+        <v>0.60416666666666663</v>
       </c>
       <c r="G220" s="12" t="s">
-        <v>295</v>
+        <v>346</v>
       </c>
       <c r="H220" s="13">
-        <v>0.36458333333333331</v>
+        <v>0.65625</v>
       </c>
       <c r="I220" s="26"/>
       <c r="J220" s="15" t="s">
         <v>358</v>
       </c>
       <c r="K220" s="22">
-        <v>27740</v>
+        <v>0</v>
       </c>
       <c r="L220" s="15"/>
       <c r="M220" s="15"/>
     </row>
     <row r="221" spans="1:13">
       <c r="A221" s="14">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="B221" s="42">
-        <v>46229</v>
+        <v>46183</v>
       </c>
       <c r="C221" s="12" t="s">
         <v>293</v>
       </c>
       <c r="D221" s="12" t="s">
-        <v>381</v>
+        <v>379</v>
       </c>
       <c r="E221" s="12" t="s">
-        <v>295</v>
+        <v>346</v>
       </c>
       <c r="F221" s="13">
-        <v>0.41666666666666669</v>
+        <v>0.72916666666666663</v>
       </c>
       <c r="G221" s="12" t="s">
         <v>294</v>
       </c>
       <c r="H221" s="13">
-        <v>0.48958333333333331</v>
+        <v>0.78125</v>
       </c>
       <c r="I221" s="26"/>
       <c r="J221" s="15" t="s">
@@ -53987,215 +53981,179 @@
       <c r="L221" s="15"/>
       <c r="M221" s="15"/>
     </row>
-    <row r="222" spans="1:13">
+    <row r="222" spans="1:13" hidden="1">
       <c r="A222" s="14">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="B222" s="42">
-        <v>46182</v>
+        <v>46170</v>
       </c>
       <c r="C222" s="12" t="s">
         <v>293</v>
       </c>
       <c r="D222" s="12" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="E222" s="12" t="s">
         <v>294</v>
       </c>
       <c r="F222" s="13">
-        <v>0.60416666666666663</v>
+        <v>0.46527777777777779</v>
       </c>
       <c r="G222" s="12" t="s">
-        <v>346</v>
+        <v>338</v>
       </c>
       <c r="H222" s="13">
-        <v>0.65625</v>
+        <v>0.52083333333333337</v>
       </c>
       <c r="I222" s="26"/>
-      <c r="J222" s="15" t="s">
-        <v>358</v>
-      </c>
+      <c r="J222" s="15"/>
       <c r="K222" s="22">
         <v>0</v>
       </c>
-      <c r="L222" s="15"/>
+      <c r="L222" s="15" t="s">
+        <v>297</v>
+      </c>
       <c r="M222" s="15"/>
     </row>
-    <row r="223" spans="1:13">
+    <row r="223" spans="1:13" hidden="1">
       <c r="A223" s="14">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="B223" s="42">
-        <v>46183</v>
+        <v>46171</v>
       </c>
       <c r="C223" s="12" t="s">
         <v>293</v>
       </c>
       <c r="D223" s="12" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="E223" s="12" t="s">
-        <v>346</v>
+        <v>338</v>
       </c>
       <c r="F223" s="13">
-        <v>0.72916666666666663</v>
+        <v>0.63541666666666663</v>
       </c>
       <c r="G223" s="12" t="s">
         <v>294</v>
       </c>
       <c r="H223" s="13">
-        <v>0.78125</v>
+        <v>0.69444444444444442</v>
       </c>
       <c r="I223" s="26"/>
-      <c r="J223" s="15" t="s">
-        <v>358</v>
-      </c>
+      <c r="J223" s="15"/>
       <c r="K223" s="22">
         <v>0</v>
       </c>
-      <c r="L223" s="15"/>
+      <c r="L223" s="15" t="s">
+        <v>297</v>
+      </c>
       <c r="M223" s="15"/>
     </row>
-    <row r="224" spans="1:13" hidden="1">
+    <row r="224" spans="1:13" ht="14.25">
       <c r="A224" s="14">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="B224" s="42">
-        <v>46170</v>
+        <v>46180</v>
       </c>
       <c r="C224" s="12" t="s">
         <v>293</v>
       </c>
       <c r="D224" s="12" t="s">
-        <v>383</v>
+        <v>374</v>
       </c>
       <c r="E224" s="12" t="s">
         <v>294</v>
       </c>
       <c r="F224" s="13">
-        <v>0.46527777777777779</v>
+        <v>0.33333333333333331</v>
       </c>
       <c r="G224" s="12" t="s">
-        <v>338</v>
+        <v>375</v>
       </c>
       <c r="H224" s="13">
-        <v>0.52083333333333337</v>
-      </c>
-      <c r="I224" s="26"/>
+        <v>0.40625</v>
+      </c>
+      <c r="I224" s="61"/>
       <c r="J224" s="15"/>
       <c r="K224" s="22">
         <v>0</v>
       </c>
-      <c r="L224" s="15" t="s">
-        <v>297</v>
-      </c>
+      <c r="L224" s="15"/>
       <c r="M224" s="15"/>
     </row>
-    <row r="225" spans="1:13" hidden="1">
+    <row r="225" spans="1:13" ht="14.25">
       <c r="A225" s="14">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="B225" s="42">
-        <v>46171</v>
+        <v>46181</v>
       </c>
       <c r="C225" s="12" t="s">
         <v>293</v>
       </c>
       <c r="D225" s="12" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="E225" s="12" t="s">
-        <v>338</v>
+        <v>375</v>
       </c>
       <c r="F225" s="13">
-        <v>0.63541666666666663</v>
+        <v>0.72222222222222221</v>
       </c>
       <c r="G225" s="12" t="s">
         <v>294</v>
       </c>
       <c r="H225" s="13">
-        <v>0.69444444444444442</v>
-      </c>
-      <c r="I225" s="26"/>
+        <v>0.79513888888888884</v>
+      </c>
+      <c r="I225" s="61"/>
       <c r="J225" s="15"/>
       <c r="K225" s="22">
         <v>0</v>
       </c>
-      <c r="L225" s="15" t="s">
-        <v>297</v>
-      </c>
+      <c r="L225" s="15"/>
       <c r="M225" s="15"/>
     </row>
     <row r="226" spans="1:13" ht="14.25">
       <c r="A226" s="14">
-        <v>236</v>
-      </c>
-      <c r="B226" s="42">
-        <v>46180</v>
-      </c>
-      <c r="C226" s="12" t="s">
-        <v>293</v>
-      </c>
-      <c r="D226" s="12" t="s">
-        <v>374</v>
-      </c>
-      <c r="E226" s="12" t="s">
-        <v>294</v>
-      </c>
-      <c r="F226" s="13">
-        <v>0.33333333333333331</v>
-      </c>
-      <c r="G226" s="12" t="s">
-        <v>375</v>
-      </c>
-      <c r="H226" s="13">
-        <v>0.40625</v>
-      </c>
+        <v>241</v>
+      </c>
+      <c r="B226" s="42"/>
+      <c r="C226" s="61"/>
+      <c r="D226" s="61"/>
+      <c r="E226" s="61"/>
+      <c r="F226" s="62"/>
+      <c r="G226" s="61"/>
+      <c r="H226" s="62"/>
       <c r="I226" s="61"/>
       <c r="J226" s="15"/>
-      <c r="K226" s="22">
-        <v>0</v>
-      </c>
+      <c r="K226" s="22"/>
       <c r="L226" s="15"/>
       <c r="M226" s="15"/>
     </row>
     <row r="227" spans="1:13" ht="14.25">
       <c r="A227" s="14">
-        <v>237</v>
-      </c>
-      <c r="B227" s="42">
-        <v>46181</v>
-      </c>
-      <c r="C227" s="12" t="s">
-        <v>293</v>
-      </c>
-      <c r="D227" s="12" t="s">
-        <v>385</v>
-      </c>
-      <c r="E227" s="12" t="s">
-        <v>375</v>
-      </c>
-      <c r="F227" s="13">
-        <v>0.72222222222222221</v>
-      </c>
-      <c r="G227" s="12" t="s">
-        <v>294</v>
-      </c>
-      <c r="H227" s="13">
-        <v>0.79513888888888884</v>
-      </c>
+        <v>242</v>
+      </c>
+      <c r="B227" s="42"/>
+      <c r="C227" s="61"/>
+      <c r="D227" s="61"/>
+      <c r="E227" s="61"/>
+      <c r="F227" s="62"/>
+      <c r="G227" s="61"/>
+      <c r="H227" s="62"/>
       <c r="I227" s="61"/>
       <c r="J227" s="15"/>
-      <c r="K227" s="22">
-        <v>0</v>
-      </c>
+      <c r="K227" s="22"/>
       <c r="L227" s="15"/>
       <c r="M227" s="15"/>
     </row>
     <row r="228" spans="1:13" ht="14.25">
       <c r="A228" s="14">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="B228" s="42"/>
       <c r="C228" s="61"/>
@@ -54212,7 +54170,7 @@
     </row>
     <row r="229" spans="1:13" ht="14.25">
       <c r="A229" s="14">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="B229" s="42"/>
       <c r="C229" s="61"/>
@@ -54229,7 +54187,7 @@
     </row>
     <row r="230" spans="1:13" ht="14.25">
       <c r="A230" s="14">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="B230" s="42"/>
       <c r="C230" s="61"/>
@@ -54246,7 +54204,7 @@
     </row>
     <row r="231" spans="1:13" ht="14.25">
       <c r="A231" s="14">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="B231" s="42"/>
       <c r="C231" s="61"/>
@@ -54263,7 +54221,7 @@
     </row>
     <row r="232" spans="1:13" ht="14.25">
       <c r="A232" s="14">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="B232" s="42"/>
       <c r="C232" s="61"/>
@@ -54280,7 +54238,7 @@
     </row>
     <row r="233" spans="1:13" ht="14.25">
       <c r="A233" s="14">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="B233" s="42"/>
       <c r="C233" s="61"/>
@@ -54297,7 +54255,7 @@
     </row>
     <row r="234" spans="1:13" ht="14.25">
       <c r="A234" s="14">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="B234" s="42"/>
       <c r="C234" s="61"/>
@@ -54314,7 +54272,7 @@
     </row>
     <row r="235" spans="1:13" ht="14.25">
       <c r="A235" s="14">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="B235" s="42"/>
       <c r="C235" s="61"/>
@@ -54331,7 +54289,7 @@
     </row>
     <row r="236" spans="1:13" ht="14.25">
       <c r="A236" s="14">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="B236" s="42"/>
       <c r="C236" s="61"/>
@@ -54348,7 +54306,7 @@
     </row>
     <row r="237" spans="1:13" ht="14.25">
       <c r="A237" s="14">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="B237" s="42"/>
       <c r="C237" s="61"/>
@@ -54365,7 +54323,7 @@
     </row>
     <row r="238" spans="1:13" ht="14.25">
       <c r="A238" s="14">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="B238" s="42"/>
       <c r="C238" s="61"/>
@@ -54382,7 +54340,7 @@
     </row>
     <row r="239" spans="1:13" ht="14.25">
       <c r="A239" s="14">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="B239" s="42"/>
       <c r="C239" s="61"/>
@@ -54399,7 +54357,7 @@
     </row>
     <row r="240" spans="1:13" ht="14.25">
       <c r="A240" s="14">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="B240" s="42"/>
       <c r="C240" s="61"/>
@@ -54416,7 +54374,7 @@
     </row>
     <row r="241" spans="1:13" ht="14.25">
       <c r="A241" s="14">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="B241" s="42"/>
       <c r="C241" s="61"/>
@@ -54433,7 +54391,7 @@
     </row>
     <row r="242" spans="1:13" ht="14.25">
       <c r="A242" s="14">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="B242" s="42"/>
       <c r="C242" s="61"/>
@@ -54450,7 +54408,7 @@
     </row>
     <row r="243" spans="1:13" ht="14.25">
       <c r="A243" s="14">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="B243" s="42"/>
       <c r="C243" s="61"/>
@@ -54467,7 +54425,7 @@
     </row>
     <row r="244" spans="1:13" ht="14.25">
       <c r="A244" s="14">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="B244" s="42"/>
       <c r="C244" s="61"/>
@@ -54484,7 +54442,7 @@
     </row>
     <row r="245" spans="1:13" ht="14.25">
       <c r="A245" s="14">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="B245" s="42"/>
       <c r="C245" s="61"/>
@@ -54501,7 +54459,7 @@
     </row>
     <row r="246" spans="1:13" ht="14.25">
       <c r="A246" s="14">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="B246" s="42"/>
       <c r="C246" s="61"/>
@@ -54518,7 +54476,7 @@
     </row>
     <row r="247" spans="1:13" ht="14.25">
       <c r="A247" s="14">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="B247" s="42"/>
       <c r="C247" s="61"/>
@@ -54535,7 +54493,7 @@
     </row>
     <row r="248" spans="1:13" ht="14.25">
       <c r="A248" s="14">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="B248" s="42"/>
       <c r="C248" s="61"/>
@@ -54552,7 +54510,7 @@
     </row>
     <row r="249" spans="1:13" ht="14.25">
       <c r="A249" s="14">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="B249" s="42"/>
       <c r="C249" s="61"/>
@@ -54569,7 +54527,7 @@
     </row>
     <row r="250" spans="1:13" ht="14.25">
       <c r="A250" s="14">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="B250" s="42"/>
       <c r="C250" s="61"/>
@@ -54586,7 +54544,7 @@
     </row>
     <row r="251" spans="1:13" ht="14.25">
       <c r="A251" s="14">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="B251" s="42"/>
       <c r="C251" s="61"/>
@@ -54603,7 +54561,7 @@
     </row>
     <row r="252" spans="1:13" ht="14.25">
       <c r="A252" s="14">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="B252" s="42"/>
       <c r="C252" s="61"/>
@@ -54620,7 +54578,7 @@
     </row>
     <row r="253" spans="1:13" ht="14.25">
       <c r="A253" s="14">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="B253" s="42"/>
       <c r="C253" s="61"/>
@@ -54637,7 +54595,7 @@
     </row>
     <row r="254" spans="1:13" ht="14.25">
       <c r="A254" s="14">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="B254" s="42"/>
       <c r="C254" s="61"/>
@@ -54654,7 +54612,7 @@
     </row>
     <row r="255" spans="1:13" ht="14.25">
       <c r="A255" s="14">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="B255" s="42"/>
       <c r="C255" s="61"/>
@@ -54671,7 +54629,7 @@
     </row>
     <row r="256" spans="1:13" ht="14.25">
       <c r="A256" s="14">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="B256" s="42"/>
       <c r="C256" s="61"/>
@@ -54688,7 +54646,7 @@
     </row>
     <row r="257" spans="1:13" ht="14.25">
       <c r="A257" s="14">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="B257" s="42"/>
       <c r="C257" s="61"/>
@@ -54705,7 +54663,7 @@
     </row>
     <row r="258" spans="1:13" ht="14.25">
       <c r="A258" s="14">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="B258" s="42"/>
       <c r="C258" s="61"/>
@@ -54722,7 +54680,7 @@
     </row>
     <row r="259" spans="1:13" ht="14.25">
       <c r="A259" s="14">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="B259" s="42"/>
       <c r="C259" s="61"/>
@@ -54739,7 +54697,7 @@
     </row>
     <row r="260" spans="1:13" ht="14.25">
       <c r="A260" s="14">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="B260" s="42"/>
       <c r="C260" s="61"/>
@@ -54750,39 +54708,39 @@
       <c r="H260" s="62"/>
       <c r="I260" s="61"/>
       <c r="J260" s="15"/>
-      <c r="K260" s="22"/>
+      <c r="K260" s="15"/>
       <c r="L260" s="15"/>
       <c r="M260" s="15"/>
     </row>
-    <row r="261" spans="1:13" ht="14.25">
+    <row r="261" spans="1:13">
       <c r="A261" s="14">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="B261" s="42"/>
-      <c r="C261" s="61"/>
-      <c r="D261" s="61"/>
-      <c r="E261" s="61"/>
-      <c r="F261" s="62"/>
-      <c r="G261" s="61"/>
-      <c r="H261" s="62"/>
-      <c r="I261" s="61"/>
+      <c r="C261" s="12"/>
+      <c r="D261" s="12"/>
+      <c r="E261" s="12"/>
+      <c r="F261" s="13"/>
+      <c r="G261" s="12"/>
+      <c r="H261" s="13"/>
+      <c r="I261" s="15"/>
       <c r="J261" s="15"/>
-      <c r="K261" s="22"/>
+      <c r="K261" s="15"/>
       <c r="L261" s="15"/>
       <c r="M261" s="15"/>
     </row>
-    <row r="262" spans="1:13" ht="14.25">
+    <row r="262" spans="1:13">
       <c r="A262" s="14">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="B262" s="42"/>
-      <c r="C262" s="61"/>
-      <c r="D262" s="61"/>
-      <c r="E262" s="61"/>
-      <c r="F262" s="62"/>
-      <c r="G262" s="61"/>
-      <c r="H262" s="62"/>
-      <c r="I262" s="61"/>
+      <c r="C262" s="12"/>
+      <c r="D262" s="12"/>
+      <c r="E262" s="12"/>
+      <c r="F262" s="13"/>
+      <c r="G262" s="12"/>
+      <c r="H262" s="13"/>
+      <c r="I262" s="15"/>
       <c r="J262" s="15"/>
       <c r="K262" s="15"/>
       <c r="L262" s="15"/>
@@ -54790,242 +54748,260 @@
     </row>
     <row r="263" spans="1:13">
       <c r="A263" s="14">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="B263" s="42"/>
-      <c r="C263" s="12"/>
-      <c r="D263" s="12"/>
-      <c r="E263" s="12"/>
-      <c r="F263" s="13"/>
-      <c r="G263" s="12"/>
-      <c r="H263" s="13"/>
-      <c r="I263" s="15"/>
-      <c r="J263" s="15"/>
-      <c r="K263" s="15"/>
-      <c r="L263" s="15"/>
-      <c r="M263" s="15"/>
-    </row>
-    <row r="264" spans="1:13">
-      <c r="A264" s="14">
-        <v>277</v>
-      </c>
-      <c r="B264" s="42"/>
-      <c r="C264" s="12"/>
-      <c r="D264" s="12"/>
-      <c r="E264" s="12"/>
-      <c r="F264" s="13"/>
-      <c r="G264" s="12"/>
-      <c r="H264" s="13"/>
-      <c r="I264" s="15"/>
-      <c r="J264" s="15"/>
-      <c r="K264" s="15"/>
-      <c r="L264" s="15"/>
-      <c r="M264" s="15"/>
-    </row>
-    <row r="265" spans="1:13">
-      <c r="A265" s="14">
-        <v>278</v>
-      </c>
-      <c r="B265" s="42"/>
-      <c r="C265" s="19"/>
-      <c r="D265" s="19"/>
-      <c r="E265" s="19"/>
-      <c r="F265" s="20"/>
-      <c r="G265" s="19"/>
-      <c r="H265" s="20"/>
-      <c r="I265" s="21"/>
-      <c r="J265" s="21"/>
-      <c r="K265" s="21"/>
-      <c r="L265" s="21"/>
-      <c r="M265" s="21"/>
+      <c r="C263" s="19"/>
+      <c r="D263" s="19"/>
+      <c r="E263" s="19"/>
+      <c r="F263" s="20"/>
+      <c r="G263" s="19"/>
+      <c r="H263" s="20"/>
+      <c r="I263" s="21"/>
+      <c r="J263" s="21"/>
+      <c r="K263" s="21"/>
+      <c r="L263" s="21"/>
+      <c r="M263" s="21"/>
+    </row>
+    <row r="274" spans="10:11">
+      <c r="J274" t="s">
+        <v>384</v>
+      </c>
+      <c r="K274" s="11">
+        <f>SUM(テーブル4[料金])</f>
+        <v>1363524</v>
+      </c>
+    </row>
+    <row r="275" spans="10:11">
+      <c r="J275" t="s">
+        <v>385</v>
+      </c>
+      <c r="K275">
+        <f>COUNTA(テーブル4[料金])*5</f>
+        <v>1100</v>
+      </c>
     </row>
     <row r="276" spans="10:11">
       <c r="J276" t="s">
-        <v>386</v>
-      </c>
-      <c r="K276" s="11">
-        <f>SUM(テーブル4[料金])</f>
-        <v>1363524</v>
+        <v>5</v>
+      </c>
+      <c r="K276">
+        <f>COUNTA(テーブル4[料金])</f>
+        <v>220</v>
       </c>
     </row>
     <row r="277" spans="10:11">
       <c r="J277" t="s">
+        <v>386</v>
+      </c>
+      <c r="K277" s="41">
+        <f>K274/K275</f>
+        <v>1239.5672727272727</v>
+      </c>
+    </row>
+    <row r="289" spans="1:8">
+      <c r="A289" s="24" t="s">
+        <v>281</v>
+      </c>
+      <c r="B289" s="24" t="s">
+        <v>282</v>
+      </c>
+      <c r="C289" s="24" t="s">
+        <v>283</v>
+      </c>
+      <c r="D289" s="24" t="s">
+        <v>284</v>
+      </c>
+      <c r="E289" s="24" t="s">
+        <v>285</v>
+      </c>
+      <c r="F289" s="24" t="s">
+        <v>286</v>
+      </c>
+      <c r="G289" s="24" t="s">
+        <v>287</v>
+      </c>
+      <c r="H289" s="24" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="290" spans="1:8">
+      <c r="A290">
+        <v>1</v>
+      </c>
+      <c r="B290" t="s">
+        <v>304</v>
+      </c>
+      <c r="C290">
+        <v>51</v>
+      </c>
+      <c r="D290" t="s">
+        <v>295</v>
+      </c>
+      <c r="E290" s="25">
+        <v>0.2986111111111111</v>
+      </c>
+      <c r="F290" t="s">
+        <v>305</v>
+      </c>
+      <c r="G290" s="25">
+        <v>0.36805555555555558</v>
+      </c>
+      <c r="H290" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="291" spans="1:8">
+      <c r="A291">
+        <v>2</v>
+      </c>
+      <c r="B291" t="s">
+        <v>309</v>
+      </c>
+      <c r="C291">
+        <v>873</v>
+      </c>
+      <c r="D291" t="s">
+        <v>305</v>
+      </c>
+      <c r="E291" s="25">
+        <v>0.41319444444444442</v>
+      </c>
+      <c r="F291" t="s">
+        <v>331</v>
+      </c>
+      <c r="G291" s="25">
+        <v>0.43402777777777779</v>
+      </c>
+      <c r="H291" t="s">
         <v>387</v>
-      </c>
-      <c r="K277">
-        <f>COUNTA(テーブル4[料金])*5</f>
-        <v>1100</v>
-      </c>
-    </row>
-    <row r="278" spans="10:11">
-      <c r="J278" t="s">
-        <v>5</v>
-      </c>
-      <c r="K278">
-        <f>COUNTA(テーブル4[料金])</f>
-        <v>220</v>
-      </c>
-    </row>
-    <row r="279" spans="10:11">
-      <c r="J279" t="s">
-        <v>388</v>
-      </c>
-      <c r="K279" s="41">
-        <f>K276/K277</f>
-        <v>1239.5672727272727</v>
-      </c>
-    </row>
-    <row r="291" spans="1:8">
-      <c r="A291" s="24" t="s">
-        <v>281</v>
-      </c>
-      <c r="B291" s="24" t="s">
-        <v>282</v>
-      </c>
-      <c r="C291" s="24" t="s">
-        <v>283</v>
-      </c>
-      <c r="D291" s="24" t="s">
-        <v>284</v>
-      </c>
-      <c r="E291" s="24" t="s">
-        <v>285</v>
-      </c>
-      <c r="F291" s="24" t="s">
-        <v>286</v>
-      </c>
-      <c r="G291" s="24" t="s">
-        <v>287</v>
-      </c>
-      <c r="H291" s="24" t="s">
-        <v>288</v>
       </c>
     </row>
     <row r="292" spans="1:8">
       <c r="A292">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B292" t="s">
-        <v>304</v>
+        <v>309</v>
       </c>
       <c r="C292">
-        <v>51</v>
+        <v>874</v>
       </c>
       <c r="D292" t="s">
-        <v>295</v>
+        <v>331</v>
       </c>
       <c r="E292" s="25">
-        <v>0.2986111111111111</v>
+        <v>0.45833333333333331</v>
       </c>
       <c r="F292" t="s">
         <v>305</v>
       </c>
       <c r="G292" s="25">
-        <v>0.36805555555555558</v>
+        <v>0.4826388888888889</v>
       </c>
       <c r="H292" t="s">
-        <v>296</v>
+        <v>301</v>
       </c>
     </row>
     <row r="293" spans="1:8">
       <c r="A293">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="B293" t="s">
-        <v>309</v>
+        <v>304</v>
       </c>
       <c r="C293">
-        <v>873</v>
+        <v>609</v>
       </c>
       <c r="D293" t="s">
         <v>305</v>
       </c>
       <c r="E293" s="25">
-        <v>0.41319444444444442</v>
+        <v>0.53472222222222221</v>
       </c>
       <c r="F293" t="s">
-        <v>331</v>
+        <v>308</v>
       </c>
       <c r="G293" s="25">
-        <v>0.43402777777777779</v>
+        <v>0.57291666666666663</v>
       </c>
       <c r="H293" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
     </row>
     <row r="294" spans="1:8">
       <c r="A294">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="B294" t="s">
-        <v>309</v>
+        <v>304</v>
       </c>
       <c r="C294">
-        <v>874</v>
+        <v>614</v>
       </c>
       <c r="D294" t="s">
-        <v>331</v>
+        <v>308</v>
       </c>
       <c r="E294" s="25">
-        <v>0.45833333333333331</v>
+        <v>0.60069444444444442</v>
       </c>
       <c r="F294" t="s">
         <v>305</v>
       </c>
       <c r="G294" s="25">
-        <v>0.4826388888888889</v>
+        <v>0.64583333333333337</v>
       </c>
       <c r="H294" t="s">
-        <v>301</v>
+        <v>306</v>
       </c>
     </row>
     <row r="295" spans="1:8">
       <c r="A295">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="B295" t="s">
         <v>304</v>
       </c>
       <c r="C295">
-        <v>609</v>
+        <v>567</v>
       </c>
       <c r="D295" t="s">
         <v>305</v>
       </c>
       <c r="E295" s="25">
-        <v>0.53472222222222221</v>
+        <v>0.67361111111111116</v>
       </c>
       <c r="F295" t="s">
-        <v>308</v>
+        <v>312</v>
       </c>
       <c r="G295" s="25">
-        <v>0.57291666666666663</v>
+        <v>0.70833333333333337</v>
       </c>
       <c r="H295" t="s">
-        <v>390</v>
+        <v>306</v>
       </c>
     </row>
     <row r="296" spans="1:8">
       <c r="A296">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="B296" t="s">
         <v>304</v>
       </c>
       <c r="C296">
-        <v>614</v>
+        <v>566</v>
       </c>
       <c r="D296" t="s">
-        <v>308</v>
+        <v>312</v>
       </c>
       <c r="E296" s="25">
-        <v>0.60069444444444442</v>
+        <v>0.73611111111111116</v>
       </c>
       <c r="F296" t="s">
         <v>305</v>
       </c>
       <c r="G296" s="25">
-        <v>0.64583333333333337</v>
+        <v>0.77430555555555558</v>
       </c>
       <c r="H296" t="s">
         <v>306</v>
@@ -55033,392 +55009,394 @@
     </row>
     <row r="297" spans="1:8">
       <c r="A297">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="B297" t="s">
-        <v>304</v>
+        <v>293</v>
       </c>
       <c r="C297">
-        <v>567</v>
+        <v>920</v>
       </c>
       <c r="D297" t="s">
         <v>305</v>
       </c>
       <c r="E297" s="25">
-        <v>0.67361111111111116</v>
+        <v>0.80902777777777779</v>
       </c>
       <c r="F297" t="s">
-        <v>312</v>
+        <v>294</v>
       </c>
       <c r="G297" s="25">
-        <v>0.70833333333333337</v>
+        <v>0.91666666666666663</v>
       </c>
       <c r="H297" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="300" spans="1:8">
+      <c r="A300" s="24" t="s">
+        <v>281</v>
+      </c>
+      <c r="B300" s="24" t="s">
+        <v>282</v>
+      </c>
+      <c r="C300" s="24" t="s">
+        <v>283</v>
+      </c>
+      <c r="D300" s="24" t="s">
+        <v>284</v>
+      </c>
+      <c r="E300" s="24" t="s">
+        <v>285</v>
+      </c>
+      <c r="F300" s="24" t="s">
+        <v>286</v>
+      </c>
+      <c r="G300" s="24" t="s">
+        <v>287</v>
+      </c>
+      <c r="H300" s="24" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="301" spans="1:8">
+      <c r="A301">
+        <v>1</v>
+      </c>
+      <c r="B301" t="s">
+        <v>304</v>
+      </c>
+      <c r="C301">
+        <v>51</v>
+      </c>
+      <c r="D301" t="s">
+        <v>295</v>
+      </c>
+      <c r="E301" s="25">
+        <v>0.2986111111111111</v>
+      </c>
+      <c r="F301" t="s">
+        <v>305</v>
+      </c>
+      <c r="G301" s="25">
+        <v>0.36805555555555558</v>
+      </c>
+      <c r="H301" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="302" spans="1:8">
+      <c r="A302">
+        <v>2</v>
+      </c>
+      <c r="B302" t="s">
+        <v>304</v>
+      </c>
+      <c r="C302">
+        <v>605</v>
+      </c>
+      <c r="D302" t="s">
+        <v>305</v>
+      </c>
+      <c r="E302" s="25">
+        <v>0.39583333333333331</v>
+      </c>
+      <c r="F302" t="s">
+        <v>308</v>
+      </c>
+      <c r="G302" s="25">
+        <v>0.43402777777777779</v>
+      </c>
+      <c r="H302" t="s">
         <v>306</v>
-      </c>
-    </row>
-    <row r="298" spans="1:8">
-      <c r="A298">
-        <v>7</v>
-      </c>
-      <c r="B298" t="s">
-        <v>304</v>
-      </c>
-      <c r="C298">
-        <v>566</v>
-      </c>
-      <c r="D298" t="s">
-        <v>312</v>
-      </c>
-      <c r="E298" s="25">
-        <v>0.73611111111111116</v>
-      </c>
-      <c r="F298" t="s">
-        <v>305</v>
-      </c>
-      <c r="G298" s="25">
-        <v>0.77430555555555558</v>
-      </c>
-      <c r="H298" t="s">
-        <v>306</v>
-      </c>
-    </row>
-    <row r="299" spans="1:8">
-      <c r="A299">
-        <v>8</v>
-      </c>
-      <c r="B299" t="s">
-        <v>293</v>
-      </c>
-      <c r="C299">
-        <v>920</v>
-      </c>
-      <c r="D299" t="s">
-        <v>305</v>
-      </c>
-      <c r="E299" s="25">
-        <v>0.80902777777777779</v>
-      </c>
-      <c r="F299" t="s">
-        <v>294</v>
-      </c>
-      <c r="G299" s="25">
-        <v>0.91666666666666663</v>
-      </c>
-      <c r="H299" t="s">
-        <v>391</v>
-      </c>
-    </row>
-    <row r="302" spans="1:8">
-      <c r="A302" s="24" t="s">
-        <v>281</v>
-      </c>
-      <c r="B302" s="24" t="s">
-        <v>282</v>
-      </c>
-      <c r="C302" s="24" t="s">
-        <v>283</v>
-      </c>
-      <c r="D302" s="24" t="s">
-        <v>284</v>
-      </c>
-      <c r="E302" s="24" t="s">
-        <v>285</v>
-      </c>
-      <c r="F302" s="24" t="s">
-        <v>286</v>
-      </c>
-      <c r="G302" s="24" t="s">
-        <v>287</v>
-      </c>
-      <c r="H302" s="24" t="s">
-        <v>288</v>
       </c>
     </row>
     <row r="303" spans="1:8">
       <c r="A303">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B303" t="s">
-        <v>304</v>
+        <v>309</v>
       </c>
       <c r="C303">
-        <v>51</v>
+        <v>743</v>
       </c>
       <c r="D303" t="s">
-        <v>295</v>
+        <v>308</v>
       </c>
       <c r="E303" s="25">
-        <v>0.2986111111111111</v>
+        <v>0.52430555555555558</v>
       </c>
       <c r="F303" t="s">
-        <v>305</v>
+        <v>310</v>
       </c>
       <c r="G303" s="25">
-        <v>0.36805555555555558</v>
+        <v>0.54513888888888884</v>
       </c>
       <c r="H303" t="s">
-        <v>296</v>
+        <v>311</v>
       </c>
     </row>
     <row r="304" spans="1:8">
       <c r="A304">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="B304" t="s">
-        <v>304</v>
+        <v>309</v>
       </c>
       <c r="C304">
-        <v>605</v>
+        <v>744</v>
       </c>
       <c r="D304" t="s">
-        <v>305</v>
+        <v>310</v>
       </c>
       <c r="E304" s="25">
-        <v>0.39583333333333331</v>
+        <v>0.56597222222222221</v>
       </c>
       <c r="F304" t="s">
         <v>308</v>
       </c>
       <c r="G304" s="25">
-        <v>0.43402777777777779</v>
+        <v>0.58680555555555558</v>
       </c>
       <c r="H304" t="s">
-        <v>306</v>
+        <v>303</v>
       </c>
     </row>
     <row r="305" spans="1:9">
       <c r="A305">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="B305" t="s">
         <v>309</v>
       </c>
       <c r="C305">
-        <v>743</v>
+        <v>834</v>
       </c>
       <c r="D305" t="s">
         <v>308</v>
       </c>
       <c r="E305" s="25">
-        <v>0.52430555555555558</v>
+        <v>0.61111111111111116</v>
       </c>
       <c r="F305" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="G305" s="25">
-        <v>0.54513888888888884</v>
+        <v>0.63194444444444442</v>
       </c>
       <c r="H305" t="s">
-        <v>311</v>
+        <v>301</v>
       </c>
     </row>
     <row r="306" spans="1:9">
       <c r="A306">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="B306" t="s">
-        <v>309</v>
+        <v>304</v>
       </c>
       <c r="C306">
-        <v>744</v>
+        <v>564</v>
       </c>
       <c r="D306" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="E306" s="25">
-        <v>0.56597222222222221</v>
+        <v>0.69791666666666663</v>
       </c>
       <c r="F306" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="G306" s="25">
-        <v>0.58680555555555558</v>
+        <v>0.73611111111111116</v>
       </c>
       <c r="H306" t="s">
-        <v>303</v>
+        <v>323</v>
       </c>
     </row>
     <row r="307" spans="1:9">
       <c r="A307">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="B307" t="s">
-        <v>309</v>
+        <v>293</v>
       </c>
       <c r="C307">
-        <v>834</v>
+        <v>920</v>
       </c>
       <c r="D307" t="s">
+        <v>305</v>
+      </c>
+      <c r="E307" s="25">
+        <v>0.80902777777777779</v>
+      </c>
+      <c r="F307" t="s">
+        <v>294</v>
+      </c>
+      <c r="G307" s="25">
+        <v>0.91666666666666663</v>
+      </c>
+      <c r="H307" t="s">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="309" spans="1:9" ht="14.25">
+      <c r="A309" s="48">
+        <v>1</v>
+      </c>
+      <c r="B309" s="49" t="s">
+        <v>293</v>
+      </c>
+      <c r="C309" s="49">
+        <v>901</v>
+      </c>
+      <c r="D309" s="49" t="s">
+        <v>294</v>
+      </c>
+      <c r="E309" s="50">
+        <v>0.27083333333333331</v>
+      </c>
+      <c r="F309" s="49" t="s">
+        <v>305</v>
+      </c>
+      <c r="G309" s="50">
+        <v>0.375</v>
+      </c>
+      <c r="H309" s="51" t="s">
+        <v>390</v>
+      </c>
+      <c r="I309" s="52"/>
+    </row>
+    <row r="310" spans="1:9" ht="14.25">
+      <c r="A310" s="53">
+        <v>2</v>
+      </c>
+      <c r="B310" s="54" t="s">
+        <v>304</v>
+      </c>
+      <c r="C310" s="54">
+        <v>605</v>
+      </c>
+      <c r="D310" s="54" t="s">
+        <v>305</v>
+      </c>
+      <c r="E310" s="55">
+        <v>0.39930555555555558</v>
+      </c>
+      <c r="F310" s="54" t="s">
         <v>308</v>
       </c>
-      <c r="E307" s="25">
-        <v>0.61111111111111116</v>
-      </c>
-      <c r="F307" t="s">
-        <v>312</v>
-      </c>
-      <c r="G307" s="25">
-        <v>0.63194444444444442</v>
-      </c>
-      <c r="H307" t="s">
+      <c r="G310" s="55">
+        <v>0.44097222222222221</v>
+      </c>
+      <c r="H310" s="54" t="s">
         <v>301</v>
       </c>
-    </row>
-    <row r="308" spans="1:9">
-      <c r="A308">
-        <v>6</v>
-      </c>
-      <c r="B308" t="s">
-        <v>304</v>
-      </c>
-      <c r="C308">
-        <v>564</v>
-      </c>
-      <c r="D308" t="s">
-        <v>312</v>
-      </c>
-      <c r="E308" s="25">
-        <v>0.69791666666666663</v>
-      </c>
-      <c r="F308" t="s">
-        <v>305</v>
-      </c>
-      <c r="G308" s="25">
-        <v>0.73611111111111116</v>
-      </c>
-      <c r="H308" t="s">
-        <v>323</v>
-      </c>
-    </row>
-    <row r="309" spans="1:9">
-      <c r="A309">
-        <v>7</v>
-      </c>
-      <c r="B309" t="s">
-        <v>293</v>
-      </c>
-      <c r="C309">
-        <v>920</v>
-      </c>
-      <c r="D309" t="s">
-        <v>305</v>
-      </c>
-      <c r="E309" s="25">
-        <v>0.80902777777777779</v>
-      </c>
-      <c r="F309" t="s">
-        <v>294</v>
-      </c>
-      <c r="G309" s="25">
-        <v>0.91666666666666663</v>
-      </c>
-      <c r="H309" t="s">
-        <v>324</v>
-      </c>
+      <c r="I310" s="56"/>
     </row>
     <row r="311" spans="1:9" ht="14.25">
       <c r="A311" s="48">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B311" s="49" t="s">
-        <v>293</v>
+        <v>309</v>
       </c>
       <c r="C311" s="49">
-        <v>901</v>
+        <v>743</v>
       </c>
       <c r="D311" s="49" t="s">
-        <v>294</v>
+        <v>308</v>
       </c>
       <c r="E311" s="50">
-        <v>0.27083333333333331</v>
+        <v>0.52430555555555558</v>
       </c>
       <c r="F311" s="49" t="s">
-        <v>305</v>
+        <v>310</v>
       </c>
       <c r="G311" s="50">
-        <v>0.375</v>
-      </c>
-      <c r="H311" s="51" t="s">
-        <v>392</v>
+        <v>0.54513888888888884</v>
+      </c>
+      <c r="H311" s="49" t="s">
+        <v>391</v>
       </c>
       <c r="I311" s="52"/>
     </row>
     <row r="312" spans="1:9" ht="14.25">
       <c r="A312" s="53">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="B312" s="54" t="s">
-        <v>304</v>
+        <v>309</v>
       </c>
       <c r="C312" s="54">
-        <v>605</v>
+        <v>744</v>
       </c>
       <c r="D312" s="54" t="s">
-        <v>305</v>
+        <v>310</v>
       </c>
       <c r="E312" s="55">
-        <v>0.39930555555555558</v>
+        <v>0.56597222222222221</v>
       </c>
       <c r="F312" s="54" t="s">
         <v>308</v>
       </c>
       <c r="G312" s="55">
-        <v>0.44097222222222221</v>
+        <v>0.58680555555555558</v>
       </c>
       <c r="H312" s="54" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="I312" s="56"/>
     </row>
     <row r="313" spans="1:9" ht="14.25">
       <c r="A313" s="48">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="B313" s="49" t="s">
         <v>309</v>
       </c>
       <c r="C313" s="49">
-        <v>743</v>
+        <v>834</v>
       </c>
       <c r="D313" s="49" t="s">
         <v>308</v>
       </c>
       <c r="E313" s="50">
-        <v>0.52430555555555558</v>
+        <v>0.61111111111111116</v>
       </c>
       <c r="F313" s="49" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="G313" s="50">
-        <v>0.54513888888888884</v>
+        <v>0.63194444444444442</v>
       </c>
       <c r="H313" s="49" t="s">
-        <v>393</v>
+        <v>301</v>
       </c>
       <c r="I313" s="52"/>
     </row>
     <row r="314" spans="1:9" ht="14.25">
       <c r="A314" s="53">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="B314" s="54" t="s">
         <v>309</v>
       </c>
       <c r="C314" s="54">
-        <v>744</v>
+        <v>897</v>
       </c>
       <c r="D314" s="54" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="E314" s="55">
-        <v>0.56597222222222221</v>
+        <v>0.65277777777777779</v>
       </c>
       <c r="F314" s="54" t="s">
-        <v>308</v>
+        <v>313</v>
       </c>
       <c r="G314" s="55">
-        <v>0.58680555555555558</v>
+        <v>0.67013888888888884</v>
       </c>
       <c r="H314" s="54" t="s">
         <v>303</v>
@@ -55427,25 +55405,25 @@
     </row>
     <row r="315" spans="1:9" ht="14.25">
       <c r="A315" s="48">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="B315" s="49" t="s">
         <v>309</v>
       </c>
       <c r="C315" s="49">
-        <v>834</v>
+        <v>898</v>
       </c>
       <c r="D315" s="49" t="s">
-        <v>308</v>
+        <v>313</v>
       </c>
       <c r="E315" s="50">
-        <v>0.61111111111111116</v>
+        <v>0.69444444444444442</v>
       </c>
       <c r="F315" s="49" t="s">
         <v>312</v>
       </c>
       <c r="G315" s="50">
-        <v>0.63194444444444442</v>
+        <v>0.71180555555555558</v>
       </c>
       <c r="H315" s="49" t="s">
         <v>301</v>
@@ -55454,111 +55432,57 @@
     </row>
     <row r="316" spans="1:9" ht="14.25">
       <c r="A316" s="53">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="B316" s="54" t="s">
-        <v>309</v>
+        <v>304</v>
       </c>
       <c r="C316" s="54">
-        <v>897</v>
+        <v>572</v>
       </c>
       <c r="D316" s="54" t="s">
         <v>312</v>
       </c>
       <c r="E316" s="55">
-        <v>0.65277777777777779</v>
+        <v>0.74652777777777779</v>
       </c>
       <c r="F316" s="54" t="s">
-        <v>313</v>
+        <v>305</v>
       </c>
       <c r="G316" s="55">
-        <v>0.67013888888888884</v>
+        <v>0.78472222222222221</v>
       </c>
       <c r="H316" s="54" t="s">
-        <v>303</v>
+        <v>389</v>
       </c>
       <c r="I316" s="56"/>
     </row>
     <row r="317" spans="1:9" ht="14.25">
-      <c r="A317" s="48">
-        <v>7</v>
-      </c>
-      <c r="B317" s="49" t="s">
-        <v>309</v>
-      </c>
-      <c r="C317" s="49">
-        <v>898</v>
-      </c>
-      <c r="D317" s="49" t="s">
-        <v>313</v>
-      </c>
-      <c r="E317" s="50">
-        <v>0.69444444444444442</v>
-      </c>
-      <c r="F317" s="49" t="s">
-        <v>312</v>
-      </c>
-      <c r="G317" s="50">
-        <v>0.71180555555555558</v>
-      </c>
-      <c r="H317" s="49" t="s">
-        <v>301</v>
-      </c>
-      <c r="I317" s="52"/>
-    </row>
-    <row r="318" spans="1:9" ht="14.25">
-      <c r="A318" s="53">
-        <v>8</v>
-      </c>
-      <c r="B318" s="54" t="s">
-        <v>304</v>
-      </c>
-      <c r="C318" s="54">
-        <v>572</v>
-      </c>
-      <c r="D318" s="54" t="s">
-        <v>312</v>
-      </c>
-      <c r="E318" s="55">
-        <v>0.74652777777777779</v>
-      </c>
-      <c r="F318" s="54" t="s">
+      <c r="A317" s="57">
+        <v>9</v>
+      </c>
+      <c r="B317" s="58" t="s">
+        <v>293</v>
+      </c>
+      <c r="C317" s="58">
+        <v>920</v>
+      </c>
+      <c r="D317" s="58" t="s">
         <v>305</v>
       </c>
-      <c r="G318" s="55">
-        <v>0.78472222222222221</v>
-      </c>
-      <c r="H318" s="54" t="s">
-        <v>391</v>
-      </c>
-      <c r="I318" s="56"/>
-    </row>
-    <row r="319" spans="1:9" ht="14.25">
-      <c r="A319" s="57">
-        <v>9</v>
-      </c>
-      <c r="B319" s="58" t="s">
-        <v>293</v>
-      </c>
-      <c r="C319" s="58">
-        <v>920</v>
-      </c>
-      <c r="D319" s="58" t="s">
-        <v>305</v>
-      </c>
-      <c r="E319" s="59">
+      <c r="E317" s="59">
         <v>0.8125</v>
       </c>
-      <c r="F319" s="58" t="s">
+      <c r="F317" s="58" t="s">
         <v>294</v>
       </c>
-      <c r="G319" s="59">
+      <c r="G317" s="59">
         <v>0.91666666666666663</v>
       </c>
-      <c r="H319" s="58" t="s">
+      <c r="H317" s="58" t="s">
         <v>306</v>
       </c>
-      <c r="I319" s="60"/>
+      <c r="I317" s="60"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Update LSP management files
</commit_message>
<xml_diff>
--- a/data/20251229_LSP管理.xlsx
+++ b/data/20251229_LSP管理.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hiraizumitatsuya/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{CBC03660-AFE8-4A7A-9052-366499B9E7DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{84726649-ED8F-45D3-B7E3-A504ADBCFE80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="33600" windowHeight="20500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="33600" windowHeight="20500" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="マイル管理" sheetId="5" r:id="rId1"/>
@@ -43183,39 +43183,448 @@
   </sheetData>
   <autoFilter ref="A1:O523" xr:uid="{2A57836D-5153-486D-8B76-48FAFDDE1EA1}"/>
   <mergeCells count="499">
-    <mergeCell ref="B722:E722"/>
-    <mergeCell ref="B723:E723"/>
-    <mergeCell ref="B724:E724"/>
-    <mergeCell ref="B725:E725"/>
-    <mergeCell ref="B704:E704"/>
-    <mergeCell ref="B726:E726"/>
-    <mergeCell ref="B713:E713"/>
-    <mergeCell ref="B714:E714"/>
-    <mergeCell ref="B715:E715"/>
-    <mergeCell ref="B716:E716"/>
-    <mergeCell ref="B717:E717"/>
-    <mergeCell ref="B718:E718"/>
-    <mergeCell ref="B719:E719"/>
-    <mergeCell ref="B720:E720"/>
-    <mergeCell ref="B721:E721"/>
-    <mergeCell ref="B703:E703"/>
-    <mergeCell ref="B706:E706"/>
-    <mergeCell ref="B707:E707"/>
-    <mergeCell ref="B708:E708"/>
-    <mergeCell ref="B709:E709"/>
-    <mergeCell ref="B710:E710"/>
-    <mergeCell ref="B711:E711"/>
-    <mergeCell ref="B712:E712"/>
-    <mergeCell ref="B693:E693"/>
-    <mergeCell ref="B677:E677"/>
-    <mergeCell ref="B678:E678"/>
-    <mergeCell ref="B680:E680"/>
-    <mergeCell ref="B681:E681"/>
-    <mergeCell ref="B682:E682"/>
-    <mergeCell ref="B683:E683"/>
-    <mergeCell ref="B684:E684"/>
-    <mergeCell ref="B685:E685"/>
-    <mergeCell ref="B686:E686"/>
+    <mergeCell ref="B651:E651"/>
+    <mergeCell ref="B695:E695"/>
+    <mergeCell ref="B696:E696"/>
+    <mergeCell ref="B697:E697"/>
+    <mergeCell ref="B698:E698"/>
+    <mergeCell ref="B699:E699"/>
+    <mergeCell ref="B701:E701"/>
+    <mergeCell ref="B657:E657"/>
+    <mergeCell ref="B658:E658"/>
+    <mergeCell ref="B659:E659"/>
+    <mergeCell ref="B660:E660"/>
+    <mergeCell ref="B667:E667"/>
+    <mergeCell ref="B668:E668"/>
+    <mergeCell ref="B669:E669"/>
+    <mergeCell ref="B670:E670"/>
+    <mergeCell ref="B671:E671"/>
+    <mergeCell ref="B672:E672"/>
+    <mergeCell ref="B673:E673"/>
+    <mergeCell ref="B674:E674"/>
+    <mergeCell ref="B675:E675"/>
+    <mergeCell ref="B687:E687"/>
+    <mergeCell ref="B688:E688"/>
+    <mergeCell ref="B691:E691"/>
+    <mergeCell ref="B692:E692"/>
+    <mergeCell ref="B601:E601"/>
+    <mergeCell ref="B602:E602"/>
+    <mergeCell ref="B603:E603"/>
+    <mergeCell ref="B604:E604"/>
+    <mergeCell ref="B620:E620"/>
+    <mergeCell ref="B626:E626"/>
+    <mergeCell ref="B653:E653"/>
+    <mergeCell ref="B654:E654"/>
+    <mergeCell ref="B655:E655"/>
+    <mergeCell ref="B636:E636"/>
+    <mergeCell ref="B637:E637"/>
+    <mergeCell ref="B638:E638"/>
+    <mergeCell ref="B639:E639"/>
+    <mergeCell ref="B640:E640"/>
+    <mergeCell ref="B641:E641"/>
+    <mergeCell ref="B652:E652"/>
+    <mergeCell ref="B642:E642"/>
+    <mergeCell ref="B643:E643"/>
+    <mergeCell ref="B644:E644"/>
+    <mergeCell ref="B645:E645"/>
+    <mergeCell ref="B646:E646"/>
+    <mergeCell ref="B648:E648"/>
+    <mergeCell ref="B649:E649"/>
+    <mergeCell ref="B650:E650"/>
+    <mergeCell ref="B551:E551"/>
+    <mergeCell ref="B552:E552"/>
+    <mergeCell ref="B553:E553"/>
+    <mergeCell ref="B557:E557"/>
+    <mergeCell ref="B561:E561"/>
+    <mergeCell ref="B562:E562"/>
+    <mergeCell ref="B563:E563"/>
+    <mergeCell ref="B606:E606"/>
+    <mergeCell ref="B599:E599"/>
+    <mergeCell ref="B595:E595"/>
+    <mergeCell ref="B596:E596"/>
+    <mergeCell ref="B597:E597"/>
+    <mergeCell ref="B598:E598"/>
+    <mergeCell ref="B558:E558"/>
+    <mergeCell ref="B559:E559"/>
+    <mergeCell ref="B556:E556"/>
+    <mergeCell ref="B605:E605"/>
+    <mergeCell ref="B567:E567"/>
+    <mergeCell ref="B564:E564"/>
+    <mergeCell ref="B565:E565"/>
+    <mergeCell ref="B566:E566"/>
+    <mergeCell ref="B575:E575"/>
+    <mergeCell ref="B577:E577"/>
+    <mergeCell ref="B579:E579"/>
+    <mergeCell ref="B528:E528"/>
+    <mergeCell ref="B529:E529"/>
+    <mergeCell ref="B530:E530"/>
+    <mergeCell ref="B531:E531"/>
+    <mergeCell ref="B532:E532"/>
+    <mergeCell ref="B367:E367"/>
+    <mergeCell ref="B370:E370"/>
+    <mergeCell ref="B506:E506"/>
+    <mergeCell ref="B507:E507"/>
+    <mergeCell ref="B508:E508"/>
+    <mergeCell ref="B509:E509"/>
+    <mergeCell ref="B510:E510"/>
+    <mergeCell ref="B371:E371"/>
+    <mergeCell ref="B410:E410"/>
+    <mergeCell ref="B408:E408"/>
+    <mergeCell ref="B374:E374"/>
+    <mergeCell ref="B436:E436"/>
+    <mergeCell ref="B449:E449"/>
+    <mergeCell ref="B459:E459"/>
+    <mergeCell ref="B460:E460"/>
+    <mergeCell ref="B461:E461"/>
+    <mergeCell ref="B465:E465"/>
+    <mergeCell ref="B478:E478"/>
+    <mergeCell ref="B479:E479"/>
+    <mergeCell ref="B375:E375"/>
+    <mergeCell ref="B376:E376"/>
+    <mergeCell ref="B319:E319"/>
+    <mergeCell ref="B303:E303"/>
+    <mergeCell ref="B304:E304"/>
+    <mergeCell ref="B306:E306"/>
+    <mergeCell ref="B307:E307"/>
+    <mergeCell ref="B308:E308"/>
+    <mergeCell ref="B309:E309"/>
+    <mergeCell ref="B311:E311"/>
+    <mergeCell ref="B312:E312"/>
+    <mergeCell ref="B313:E313"/>
+    <mergeCell ref="B314:E314"/>
+    <mergeCell ref="B315:E315"/>
+    <mergeCell ref="B316:E316"/>
+    <mergeCell ref="B317:E317"/>
+    <mergeCell ref="B318:E318"/>
+    <mergeCell ref="B325:E325"/>
+    <mergeCell ref="B329:E329"/>
+    <mergeCell ref="B333:E333"/>
+    <mergeCell ref="B342:E342"/>
+    <mergeCell ref="B347:E347"/>
+    <mergeCell ref="B361:E361"/>
+    <mergeCell ref="B368:E368"/>
+    <mergeCell ref="B369:E369"/>
+    <mergeCell ref="B320:E320"/>
+    <mergeCell ref="B321:E321"/>
+    <mergeCell ref="B322:E322"/>
+    <mergeCell ref="B323:E323"/>
+    <mergeCell ref="B324:E324"/>
+    <mergeCell ref="B360:E360"/>
+    <mergeCell ref="B362:E362"/>
+    <mergeCell ref="B364:E364"/>
+    <mergeCell ref="B365:E365"/>
+    <mergeCell ref="B327:E327"/>
+    <mergeCell ref="B328:E328"/>
+    <mergeCell ref="B332:E332"/>
+    <mergeCell ref="B356:E356"/>
+    <mergeCell ref="B357:E357"/>
+    <mergeCell ref="B358:E358"/>
+    <mergeCell ref="B359:E359"/>
+    <mergeCell ref="B293:E293"/>
+    <mergeCell ref="B294:E294"/>
+    <mergeCell ref="B295:E295"/>
+    <mergeCell ref="B296:E296"/>
+    <mergeCell ref="B297:E297"/>
+    <mergeCell ref="B299:E299"/>
+    <mergeCell ref="B300:E300"/>
+    <mergeCell ref="B301:E301"/>
+    <mergeCell ref="B302:E302"/>
+    <mergeCell ref="B172:E172"/>
+    <mergeCell ref="B174:E174"/>
+    <mergeCell ref="B175:E175"/>
+    <mergeCell ref="B176:E176"/>
+    <mergeCell ref="B178:E178"/>
+    <mergeCell ref="B179:E179"/>
+    <mergeCell ref="B187:E187"/>
+    <mergeCell ref="B188:E188"/>
+    <mergeCell ref="B217:E217"/>
+    <mergeCell ref="B207:E207"/>
+    <mergeCell ref="B209:E209"/>
+    <mergeCell ref="B210:E210"/>
+    <mergeCell ref="B212:E212"/>
+    <mergeCell ref="B214:E214"/>
+    <mergeCell ref="B215:E215"/>
+    <mergeCell ref="B216:E216"/>
+    <mergeCell ref="B189:E189"/>
+    <mergeCell ref="B190:E190"/>
+    <mergeCell ref="B191:E191"/>
+    <mergeCell ref="B193:E193"/>
+    <mergeCell ref="B194:E194"/>
+    <mergeCell ref="B195:E195"/>
+    <mergeCell ref="B196:E196"/>
+    <mergeCell ref="B197:E197"/>
+    <mergeCell ref="B147:E147"/>
+    <mergeCell ref="B148:E148"/>
+    <mergeCell ref="B149:E149"/>
+    <mergeCell ref="B157:E157"/>
+    <mergeCell ref="B167:E167"/>
+    <mergeCell ref="B168:E168"/>
+    <mergeCell ref="B169:E169"/>
+    <mergeCell ref="B170:E170"/>
+    <mergeCell ref="B171:E171"/>
+    <mergeCell ref="B146:E146"/>
+    <mergeCell ref="B112:E112"/>
+    <mergeCell ref="B120:E120"/>
+    <mergeCell ref="B121:E121"/>
+    <mergeCell ref="B114:E114"/>
+    <mergeCell ref="B115:E115"/>
+    <mergeCell ref="B117:E117"/>
+    <mergeCell ref="B118:E118"/>
+    <mergeCell ref="B119:E119"/>
+    <mergeCell ref="B127:E127"/>
+    <mergeCell ref="B142:E142"/>
+    <mergeCell ref="B143:E143"/>
+    <mergeCell ref="B144:E144"/>
+    <mergeCell ref="B137:E137"/>
+    <mergeCell ref="B138:E138"/>
+    <mergeCell ref="B139:E139"/>
+    <mergeCell ref="B140:E140"/>
+    <mergeCell ref="B141:E141"/>
+    <mergeCell ref="B128:E128"/>
+    <mergeCell ref="B129:E129"/>
+    <mergeCell ref="B130:E130"/>
+    <mergeCell ref="B131:E131"/>
+    <mergeCell ref="B132:E132"/>
+    <mergeCell ref="B134:E134"/>
+    <mergeCell ref="B104:E104"/>
+    <mergeCell ref="B105:E105"/>
+    <mergeCell ref="B106:E106"/>
+    <mergeCell ref="B107:E107"/>
+    <mergeCell ref="B108:E108"/>
+    <mergeCell ref="B109:E109"/>
+    <mergeCell ref="B110:E110"/>
+    <mergeCell ref="B111:E111"/>
+    <mergeCell ref="B145:E145"/>
+    <mergeCell ref="B135:E135"/>
+    <mergeCell ref="B122:E122"/>
+    <mergeCell ref="B123:E123"/>
+    <mergeCell ref="B124:E124"/>
+    <mergeCell ref="B125:E125"/>
+    <mergeCell ref="B126:E126"/>
+    <mergeCell ref="B72:E72"/>
+    <mergeCell ref="B74:E74"/>
+    <mergeCell ref="B76:E76"/>
+    <mergeCell ref="B77:E77"/>
+    <mergeCell ref="B66:E66"/>
+    <mergeCell ref="B67:E67"/>
+    <mergeCell ref="B68:E68"/>
+    <mergeCell ref="B69:E69"/>
+    <mergeCell ref="B70:E70"/>
+    <mergeCell ref="B78:E78"/>
+    <mergeCell ref="B40:E40"/>
+    <mergeCell ref="B41:E41"/>
+    <mergeCell ref="B42:E42"/>
+    <mergeCell ref="B43:E43"/>
+    <mergeCell ref="B44:E44"/>
+    <mergeCell ref="B29:E29"/>
+    <mergeCell ref="B30:E30"/>
+    <mergeCell ref="B31:E31"/>
+    <mergeCell ref="B32:E32"/>
+    <mergeCell ref="B33:E33"/>
+    <mergeCell ref="B34:E34"/>
+    <mergeCell ref="B60:E60"/>
+    <mergeCell ref="B38:E38"/>
+    <mergeCell ref="B49:E49"/>
+    <mergeCell ref="B50:E50"/>
+    <mergeCell ref="B51:E51"/>
+    <mergeCell ref="B52:E52"/>
+    <mergeCell ref="B47:E47"/>
+    <mergeCell ref="B48:E48"/>
+    <mergeCell ref="B45:E45"/>
+    <mergeCell ref="B46:E46"/>
+    <mergeCell ref="B39:E39"/>
+    <mergeCell ref="B71:E71"/>
+    <mergeCell ref="B103:E103"/>
+    <mergeCell ref="B84:E84"/>
+    <mergeCell ref="B85:E85"/>
+    <mergeCell ref="B86:E86"/>
+    <mergeCell ref="B87:E87"/>
+    <mergeCell ref="B88:E88"/>
+    <mergeCell ref="B10:E10"/>
+    <mergeCell ref="B35:E35"/>
+    <mergeCell ref="B36:E36"/>
+    <mergeCell ref="B37:E37"/>
+    <mergeCell ref="B53:E53"/>
+    <mergeCell ref="B61:E61"/>
+    <mergeCell ref="B62:E62"/>
+    <mergeCell ref="B63:E63"/>
+    <mergeCell ref="B65:E65"/>
+    <mergeCell ref="B54:E54"/>
+    <mergeCell ref="B55:E55"/>
+    <mergeCell ref="B57:E57"/>
+    <mergeCell ref="B58:E58"/>
+    <mergeCell ref="B59:E59"/>
+    <mergeCell ref="B81:E81"/>
+    <mergeCell ref="B82:E82"/>
+    <mergeCell ref="B83:E83"/>
+    <mergeCell ref="B101:E101"/>
+    <mergeCell ref="B102:E102"/>
+    <mergeCell ref="B94:E94"/>
+    <mergeCell ref="B95:E95"/>
+    <mergeCell ref="B96:E96"/>
+    <mergeCell ref="B98:E98"/>
+    <mergeCell ref="B100:E100"/>
+    <mergeCell ref="B89:E89"/>
+    <mergeCell ref="B90:E90"/>
+    <mergeCell ref="B91:E91"/>
+    <mergeCell ref="B92:E92"/>
+    <mergeCell ref="B93:E93"/>
+    <mergeCell ref="B198:E198"/>
+    <mergeCell ref="B201:E201"/>
+    <mergeCell ref="B202:E202"/>
+    <mergeCell ref="B203:E203"/>
+    <mergeCell ref="B204:E204"/>
+    <mergeCell ref="B205:E205"/>
+    <mergeCell ref="B206:E206"/>
+    <mergeCell ref="B224:E224"/>
+    <mergeCell ref="B225:E225"/>
+    <mergeCell ref="B226:E226"/>
+    <mergeCell ref="B227:E227"/>
+    <mergeCell ref="B228:E228"/>
+    <mergeCell ref="B218:E218"/>
+    <mergeCell ref="B219:E219"/>
+    <mergeCell ref="B220:E220"/>
+    <mergeCell ref="B221:E221"/>
+    <mergeCell ref="B222:E222"/>
+    <mergeCell ref="B223:E223"/>
+    <mergeCell ref="B260:E260"/>
+    <mergeCell ref="B261:E261"/>
+    <mergeCell ref="B241:E241"/>
+    <mergeCell ref="B242:E242"/>
+    <mergeCell ref="B245:E245"/>
+    <mergeCell ref="B247:E247"/>
+    <mergeCell ref="B248:E248"/>
+    <mergeCell ref="B229:E229"/>
+    <mergeCell ref="B230:E230"/>
+    <mergeCell ref="B231:E231"/>
+    <mergeCell ref="B232:E232"/>
+    <mergeCell ref="B233:E233"/>
+    <mergeCell ref="B234:E234"/>
+    <mergeCell ref="B235:E235"/>
+    <mergeCell ref="B236:E236"/>
+    <mergeCell ref="B237:E237"/>
+    <mergeCell ref="B238:E238"/>
+    <mergeCell ref="B239:E239"/>
+    <mergeCell ref="B240:E240"/>
+    <mergeCell ref="B250:E250"/>
+    <mergeCell ref="B251:E251"/>
+    <mergeCell ref="B253:E253"/>
+    <mergeCell ref="B255:E255"/>
+    <mergeCell ref="B257:E257"/>
+    <mergeCell ref="B259:E259"/>
+    <mergeCell ref="B412:E412"/>
+    <mergeCell ref="B419:E419"/>
+    <mergeCell ref="B425:E425"/>
+    <mergeCell ref="B452:E452"/>
+    <mergeCell ref="B262:E262"/>
+    <mergeCell ref="B264:E264"/>
+    <mergeCell ref="B266:E266"/>
+    <mergeCell ref="B276:E276"/>
+    <mergeCell ref="B277:E277"/>
+    <mergeCell ref="B278:E278"/>
+    <mergeCell ref="B279:E279"/>
+    <mergeCell ref="B280:E280"/>
+    <mergeCell ref="B281:E281"/>
+    <mergeCell ref="B282:E282"/>
+    <mergeCell ref="B283:E283"/>
+    <mergeCell ref="B284:E284"/>
+    <mergeCell ref="B285:E285"/>
+    <mergeCell ref="B286:E286"/>
+    <mergeCell ref="B287:E287"/>
+    <mergeCell ref="B288:E288"/>
+    <mergeCell ref="B289:E289"/>
+    <mergeCell ref="B290:E290"/>
+    <mergeCell ref="B291:E291"/>
+    <mergeCell ref="B292:E292"/>
+    <mergeCell ref="B458:E458"/>
+    <mergeCell ref="B466:E466"/>
+    <mergeCell ref="B467:E467"/>
+    <mergeCell ref="B468:E468"/>
+    <mergeCell ref="B426:E426"/>
+    <mergeCell ref="B438:E438"/>
+    <mergeCell ref="B439:E439"/>
+    <mergeCell ref="B453:E453"/>
+    <mergeCell ref="B454:E454"/>
+    <mergeCell ref="B455:E455"/>
+    <mergeCell ref="B456:E456"/>
+    <mergeCell ref="B457:E457"/>
+    <mergeCell ref="B442:E442"/>
+    <mergeCell ref="B450:E450"/>
+    <mergeCell ref="B451:E451"/>
+    <mergeCell ref="B387:E387"/>
+    <mergeCell ref="B389:E389"/>
+    <mergeCell ref="B390:E390"/>
+    <mergeCell ref="B392:E392"/>
+    <mergeCell ref="B403:E403"/>
+    <mergeCell ref="B404:E404"/>
+    <mergeCell ref="B406:E406"/>
+    <mergeCell ref="B409:E409"/>
+    <mergeCell ref="B377:E377"/>
+    <mergeCell ref="B378:E378"/>
+    <mergeCell ref="B379:E379"/>
+    <mergeCell ref="B388:E388"/>
+    <mergeCell ref="B395:E395"/>
+    <mergeCell ref="B400:E400"/>
+    <mergeCell ref="B402:E402"/>
+    <mergeCell ref="B393:E393"/>
+    <mergeCell ref="B396:E396"/>
+    <mergeCell ref="B398:E398"/>
+    <mergeCell ref="B399:E399"/>
+    <mergeCell ref="B401:E401"/>
+    <mergeCell ref="B386:E386"/>
+    <mergeCell ref="B505:E505"/>
+    <mergeCell ref="B480:E480"/>
+    <mergeCell ref="B469:E469"/>
+    <mergeCell ref="B481:E481"/>
+    <mergeCell ref="B490:E490"/>
+    <mergeCell ref="B491:E491"/>
+    <mergeCell ref="B492:E492"/>
+    <mergeCell ref="B493:E493"/>
+    <mergeCell ref="B494:E494"/>
+    <mergeCell ref="B498:E498"/>
+    <mergeCell ref="B499:E499"/>
+    <mergeCell ref="B500:E500"/>
+    <mergeCell ref="B501:E501"/>
+    <mergeCell ref="B502:E502"/>
+    <mergeCell ref="B503:E503"/>
+    <mergeCell ref="B504:E504"/>
+    <mergeCell ref="B482:E482"/>
+    <mergeCell ref="B495:E495"/>
+    <mergeCell ref="B511:E511"/>
+    <mergeCell ref="B512:E512"/>
+    <mergeCell ref="B513:E513"/>
+    <mergeCell ref="B514:E514"/>
+    <mergeCell ref="B515:E515"/>
+    <mergeCell ref="B535:E535"/>
+    <mergeCell ref="B537:E537"/>
+    <mergeCell ref="B555:E555"/>
+    <mergeCell ref="B560:E560"/>
+    <mergeCell ref="B548:E548"/>
+    <mergeCell ref="B549:E549"/>
+    <mergeCell ref="B546:E546"/>
+    <mergeCell ref="B547:E547"/>
+    <mergeCell ref="B533:E533"/>
+    <mergeCell ref="B534:E534"/>
+    <mergeCell ref="B536:E536"/>
+    <mergeCell ref="B538:E538"/>
+    <mergeCell ref="B539:E539"/>
+    <mergeCell ref="B540:E540"/>
+    <mergeCell ref="B541:E541"/>
+    <mergeCell ref="B543:E543"/>
+    <mergeCell ref="B544:E544"/>
+    <mergeCell ref="B526:E526"/>
+    <mergeCell ref="B527:E527"/>
+    <mergeCell ref="B569:E569"/>
+    <mergeCell ref="B570:E570"/>
+    <mergeCell ref="B571:E571"/>
+    <mergeCell ref="B572:E572"/>
+    <mergeCell ref="B573:E573"/>
+    <mergeCell ref="B576:E576"/>
+    <mergeCell ref="B578:E578"/>
+    <mergeCell ref="B591:E591"/>
+    <mergeCell ref="B592:E592"/>
+    <mergeCell ref="B580:E580"/>
+    <mergeCell ref="B589:E589"/>
     <mergeCell ref="B594:E594"/>
     <mergeCell ref="B627:E627"/>
     <mergeCell ref="B647:E647"/>
@@ -43240,448 +43649,39 @@
     <mergeCell ref="B624:E624"/>
     <mergeCell ref="B625:E625"/>
     <mergeCell ref="B600:E600"/>
-    <mergeCell ref="B569:E569"/>
-    <mergeCell ref="B570:E570"/>
-    <mergeCell ref="B571:E571"/>
-    <mergeCell ref="B572:E572"/>
-    <mergeCell ref="B573:E573"/>
-    <mergeCell ref="B576:E576"/>
-    <mergeCell ref="B578:E578"/>
-    <mergeCell ref="B591:E591"/>
-    <mergeCell ref="B592:E592"/>
-    <mergeCell ref="B580:E580"/>
-    <mergeCell ref="B589:E589"/>
-    <mergeCell ref="B511:E511"/>
-    <mergeCell ref="B512:E512"/>
-    <mergeCell ref="B513:E513"/>
-    <mergeCell ref="B514:E514"/>
-    <mergeCell ref="B515:E515"/>
-    <mergeCell ref="B535:E535"/>
-    <mergeCell ref="B537:E537"/>
-    <mergeCell ref="B555:E555"/>
-    <mergeCell ref="B560:E560"/>
-    <mergeCell ref="B548:E548"/>
-    <mergeCell ref="B549:E549"/>
-    <mergeCell ref="B546:E546"/>
-    <mergeCell ref="B547:E547"/>
-    <mergeCell ref="B533:E533"/>
-    <mergeCell ref="B534:E534"/>
-    <mergeCell ref="B536:E536"/>
-    <mergeCell ref="B538:E538"/>
-    <mergeCell ref="B539:E539"/>
-    <mergeCell ref="B540:E540"/>
-    <mergeCell ref="B541:E541"/>
-    <mergeCell ref="B543:E543"/>
-    <mergeCell ref="B544:E544"/>
-    <mergeCell ref="B526:E526"/>
-    <mergeCell ref="B527:E527"/>
-    <mergeCell ref="B505:E505"/>
-    <mergeCell ref="B480:E480"/>
-    <mergeCell ref="B469:E469"/>
-    <mergeCell ref="B481:E481"/>
-    <mergeCell ref="B490:E490"/>
-    <mergeCell ref="B491:E491"/>
-    <mergeCell ref="B492:E492"/>
-    <mergeCell ref="B493:E493"/>
-    <mergeCell ref="B494:E494"/>
-    <mergeCell ref="B498:E498"/>
-    <mergeCell ref="B499:E499"/>
-    <mergeCell ref="B500:E500"/>
-    <mergeCell ref="B501:E501"/>
-    <mergeCell ref="B502:E502"/>
-    <mergeCell ref="B503:E503"/>
-    <mergeCell ref="B504:E504"/>
-    <mergeCell ref="B482:E482"/>
-    <mergeCell ref="B495:E495"/>
-    <mergeCell ref="B377:E377"/>
-    <mergeCell ref="B378:E378"/>
-    <mergeCell ref="B379:E379"/>
-    <mergeCell ref="B388:E388"/>
-    <mergeCell ref="B395:E395"/>
-    <mergeCell ref="B400:E400"/>
-    <mergeCell ref="B402:E402"/>
-    <mergeCell ref="B393:E393"/>
-    <mergeCell ref="B396:E396"/>
-    <mergeCell ref="B398:E398"/>
-    <mergeCell ref="B399:E399"/>
-    <mergeCell ref="B401:E401"/>
-    <mergeCell ref="B386:E386"/>
-    <mergeCell ref="B292:E292"/>
-    <mergeCell ref="B458:E458"/>
-    <mergeCell ref="B466:E466"/>
-    <mergeCell ref="B467:E467"/>
-    <mergeCell ref="B468:E468"/>
-    <mergeCell ref="B426:E426"/>
-    <mergeCell ref="B438:E438"/>
-    <mergeCell ref="B439:E439"/>
-    <mergeCell ref="B453:E453"/>
-    <mergeCell ref="B454:E454"/>
-    <mergeCell ref="B455:E455"/>
-    <mergeCell ref="B456:E456"/>
-    <mergeCell ref="B457:E457"/>
-    <mergeCell ref="B442:E442"/>
-    <mergeCell ref="B450:E450"/>
-    <mergeCell ref="B451:E451"/>
-    <mergeCell ref="B387:E387"/>
-    <mergeCell ref="B389:E389"/>
-    <mergeCell ref="B390:E390"/>
-    <mergeCell ref="B392:E392"/>
-    <mergeCell ref="B403:E403"/>
-    <mergeCell ref="B404:E404"/>
-    <mergeCell ref="B406:E406"/>
-    <mergeCell ref="B409:E409"/>
-    <mergeCell ref="B259:E259"/>
-    <mergeCell ref="B412:E412"/>
-    <mergeCell ref="B419:E419"/>
-    <mergeCell ref="B425:E425"/>
-    <mergeCell ref="B452:E452"/>
-    <mergeCell ref="B262:E262"/>
-    <mergeCell ref="B264:E264"/>
-    <mergeCell ref="B266:E266"/>
-    <mergeCell ref="B276:E276"/>
-    <mergeCell ref="B277:E277"/>
-    <mergeCell ref="B278:E278"/>
-    <mergeCell ref="B279:E279"/>
-    <mergeCell ref="B280:E280"/>
-    <mergeCell ref="B281:E281"/>
-    <mergeCell ref="B282:E282"/>
-    <mergeCell ref="B283:E283"/>
-    <mergeCell ref="B284:E284"/>
-    <mergeCell ref="B285:E285"/>
-    <mergeCell ref="B286:E286"/>
-    <mergeCell ref="B287:E287"/>
-    <mergeCell ref="B288:E288"/>
-    <mergeCell ref="B289:E289"/>
-    <mergeCell ref="B290:E290"/>
-    <mergeCell ref="B291:E291"/>
-    <mergeCell ref="B260:E260"/>
-    <mergeCell ref="B261:E261"/>
-    <mergeCell ref="B241:E241"/>
-    <mergeCell ref="B242:E242"/>
-    <mergeCell ref="B245:E245"/>
-    <mergeCell ref="B247:E247"/>
-    <mergeCell ref="B248:E248"/>
-    <mergeCell ref="B229:E229"/>
-    <mergeCell ref="B230:E230"/>
-    <mergeCell ref="B231:E231"/>
-    <mergeCell ref="B232:E232"/>
-    <mergeCell ref="B233:E233"/>
-    <mergeCell ref="B234:E234"/>
-    <mergeCell ref="B235:E235"/>
-    <mergeCell ref="B236:E236"/>
-    <mergeCell ref="B237:E237"/>
-    <mergeCell ref="B238:E238"/>
-    <mergeCell ref="B239:E239"/>
-    <mergeCell ref="B240:E240"/>
-    <mergeCell ref="B250:E250"/>
-    <mergeCell ref="B251:E251"/>
-    <mergeCell ref="B253:E253"/>
-    <mergeCell ref="B255:E255"/>
-    <mergeCell ref="B257:E257"/>
-    <mergeCell ref="B226:E226"/>
-    <mergeCell ref="B227:E227"/>
-    <mergeCell ref="B228:E228"/>
-    <mergeCell ref="B218:E218"/>
-    <mergeCell ref="B219:E219"/>
-    <mergeCell ref="B220:E220"/>
-    <mergeCell ref="B221:E221"/>
-    <mergeCell ref="B222:E222"/>
-    <mergeCell ref="B223:E223"/>
-    <mergeCell ref="B198:E198"/>
-    <mergeCell ref="B201:E201"/>
-    <mergeCell ref="B202:E202"/>
-    <mergeCell ref="B203:E203"/>
-    <mergeCell ref="B204:E204"/>
-    <mergeCell ref="B205:E205"/>
-    <mergeCell ref="B206:E206"/>
-    <mergeCell ref="B224:E224"/>
-    <mergeCell ref="B225:E225"/>
-    <mergeCell ref="B102:E102"/>
-    <mergeCell ref="B94:E94"/>
-    <mergeCell ref="B95:E95"/>
-    <mergeCell ref="B96:E96"/>
-    <mergeCell ref="B98:E98"/>
-    <mergeCell ref="B100:E100"/>
-    <mergeCell ref="B89:E89"/>
-    <mergeCell ref="B90:E90"/>
-    <mergeCell ref="B91:E91"/>
-    <mergeCell ref="B92:E92"/>
-    <mergeCell ref="B93:E93"/>
-    <mergeCell ref="B103:E103"/>
-    <mergeCell ref="B84:E84"/>
-    <mergeCell ref="B85:E85"/>
-    <mergeCell ref="B86:E86"/>
-    <mergeCell ref="B87:E87"/>
-    <mergeCell ref="B88:E88"/>
-    <mergeCell ref="B10:E10"/>
-    <mergeCell ref="B35:E35"/>
-    <mergeCell ref="B36:E36"/>
-    <mergeCell ref="B37:E37"/>
-    <mergeCell ref="B53:E53"/>
-    <mergeCell ref="B61:E61"/>
-    <mergeCell ref="B62:E62"/>
-    <mergeCell ref="B63:E63"/>
-    <mergeCell ref="B65:E65"/>
-    <mergeCell ref="B54:E54"/>
-    <mergeCell ref="B55:E55"/>
-    <mergeCell ref="B57:E57"/>
-    <mergeCell ref="B58:E58"/>
-    <mergeCell ref="B59:E59"/>
-    <mergeCell ref="B81:E81"/>
-    <mergeCell ref="B82:E82"/>
-    <mergeCell ref="B83:E83"/>
-    <mergeCell ref="B101:E101"/>
-    <mergeCell ref="B78:E78"/>
-    <mergeCell ref="B40:E40"/>
-    <mergeCell ref="B41:E41"/>
-    <mergeCell ref="B42:E42"/>
-    <mergeCell ref="B43:E43"/>
-    <mergeCell ref="B44:E44"/>
-    <mergeCell ref="B29:E29"/>
-    <mergeCell ref="B30:E30"/>
-    <mergeCell ref="B31:E31"/>
-    <mergeCell ref="B32:E32"/>
-    <mergeCell ref="B33:E33"/>
-    <mergeCell ref="B34:E34"/>
-    <mergeCell ref="B60:E60"/>
-    <mergeCell ref="B38:E38"/>
-    <mergeCell ref="B49:E49"/>
-    <mergeCell ref="B50:E50"/>
-    <mergeCell ref="B51:E51"/>
-    <mergeCell ref="B52:E52"/>
-    <mergeCell ref="B47:E47"/>
-    <mergeCell ref="B48:E48"/>
-    <mergeCell ref="B45:E45"/>
-    <mergeCell ref="B46:E46"/>
-    <mergeCell ref="B39:E39"/>
-    <mergeCell ref="B71:E71"/>
-    <mergeCell ref="B72:E72"/>
-    <mergeCell ref="B74:E74"/>
-    <mergeCell ref="B76:E76"/>
-    <mergeCell ref="B77:E77"/>
-    <mergeCell ref="B66:E66"/>
-    <mergeCell ref="B67:E67"/>
-    <mergeCell ref="B68:E68"/>
-    <mergeCell ref="B69:E69"/>
-    <mergeCell ref="B70:E70"/>
-    <mergeCell ref="B104:E104"/>
-    <mergeCell ref="B105:E105"/>
-    <mergeCell ref="B106:E106"/>
-    <mergeCell ref="B107:E107"/>
-    <mergeCell ref="B108:E108"/>
-    <mergeCell ref="B109:E109"/>
-    <mergeCell ref="B110:E110"/>
-    <mergeCell ref="B111:E111"/>
-    <mergeCell ref="B145:E145"/>
-    <mergeCell ref="B135:E135"/>
-    <mergeCell ref="B122:E122"/>
-    <mergeCell ref="B123:E123"/>
-    <mergeCell ref="B124:E124"/>
-    <mergeCell ref="B125:E125"/>
-    <mergeCell ref="B126:E126"/>
-    <mergeCell ref="B146:E146"/>
-    <mergeCell ref="B112:E112"/>
-    <mergeCell ref="B120:E120"/>
-    <mergeCell ref="B121:E121"/>
-    <mergeCell ref="B114:E114"/>
-    <mergeCell ref="B115:E115"/>
-    <mergeCell ref="B117:E117"/>
-    <mergeCell ref="B118:E118"/>
-    <mergeCell ref="B119:E119"/>
-    <mergeCell ref="B127:E127"/>
-    <mergeCell ref="B142:E142"/>
-    <mergeCell ref="B143:E143"/>
-    <mergeCell ref="B144:E144"/>
-    <mergeCell ref="B137:E137"/>
-    <mergeCell ref="B138:E138"/>
-    <mergeCell ref="B139:E139"/>
-    <mergeCell ref="B140:E140"/>
-    <mergeCell ref="B141:E141"/>
-    <mergeCell ref="B128:E128"/>
-    <mergeCell ref="B129:E129"/>
-    <mergeCell ref="B130:E130"/>
-    <mergeCell ref="B131:E131"/>
-    <mergeCell ref="B132:E132"/>
-    <mergeCell ref="B134:E134"/>
-    <mergeCell ref="B147:E147"/>
-    <mergeCell ref="B148:E148"/>
-    <mergeCell ref="B149:E149"/>
-    <mergeCell ref="B157:E157"/>
-    <mergeCell ref="B167:E167"/>
-    <mergeCell ref="B168:E168"/>
-    <mergeCell ref="B169:E169"/>
-    <mergeCell ref="B170:E170"/>
-    <mergeCell ref="B171:E171"/>
-    <mergeCell ref="B172:E172"/>
-    <mergeCell ref="B174:E174"/>
-    <mergeCell ref="B175:E175"/>
-    <mergeCell ref="B176:E176"/>
-    <mergeCell ref="B178:E178"/>
-    <mergeCell ref="B179:E179"/>
-    <mergeCell ref="B187:E187"/>
-    <mergeCell ref="B188:E188"/>
-    <mergeCell ref="B217:E217"/>
-    <mergeCell ref="B207:E207"/>
-    <mergeCell ref="B209:E209"/>
-    <mergeCell ref="B210:E210"/>
-    <mergeCell ref="B212:E212"/>
-    <mergeCell ref="B214:E214"/>
-    <mergeCell ref="B215:E215"/>
-    <mergeCell ref="B216:E216"/>
-    <mergeCell ref="B189:E189"/>
-    <mergeCell ref="B190:E190"/>
-    <mergeCell ref="B191:E191"/>
-    <mergeCell ref="B193:E193"/>
-    <mergeCell ref="B194:E194"/>
-    <mergeCell ref="B195:E195"/>
-    <mergeCell ref="B196:E196"/>
-    <mergeCell ref="B197:E197"/>
-    <mergeCell ref="B293:E293"/>
-    <mergeCell ref="B294:E294"/>
-    <mergeCell ref="B295:E295"/>
-    <mergeCell ref="B296:E296"/>
-    <mergeCell ref="B297:E297"/>
-    <mergeCell ref="B299:E299"/>
-    <mergeCell ref="B300:E300"/>
-    <mergeCell ref="B301:E301"/>
-    <mergeCell ref="B302:E302"/>
-    <mergeCell ref="B369:E369"/>
-    <mergeCell ref="B320:E320"/>
-    <mergeCell ref="B321:E321"/>
-    <mergeCell ref="B322:E322"/>
-    <mergeCell ref="B323:E323"/>
-    <mergeCell ref="B324:E324"/>
-    <mergeCell ref="B360:E360"/>
-    <mergeCell ref="B362:E362"/>
-    <mergeCell ref="B364:E364"/>
-    <mergeCell ref="B365:E365"/>
-    <mergeCell ref="B327:E327"/>
-    <mergeCell ref="B328:E328"/>
-    <mergeCell ref="B332:E332"/>
-    <mergeCell ref="B356:E356"/>
-    <mergeCell ref="B357:E357"/>
-    <mergeCell ref="B358:E358"/>
-    <mergeCell ref="B359:E359"/>
-    <mergeCell ref="B375:E375"/>
-    <mergeCell ref="B376:E376"/>
-    <mergeCell ref="B319:E319"/>
-    <mergeCell ref="B303:E303"/>
-    <mergeCell ref="B304:E304"/>
-    <mergeCell ref="B306:E306"/>
-    <mergeCell ref="B307:E307"/>
-    <mergeCell ref="B308:E308"/>
-    <mergeCell ref="B309:E309"/>
-    <mergeCell ref="B311:E311"/>
-    <mergeCell ref="B312:E312"/>
-    <mergeCell ref="B313:E313"/>
-    <mergeCell ref="B314:E314"/>
-    <mergeCell ref="B315:E315"/>
-    <mergeCell ref="B316:E316"/>
-    <mergeCell ref="B317:E317"/>
-    <mergeCell ref="B318:E318"/>
-    <mergeCell ref="B325:E325"/>
-    <mergeCell ref="B329:E329"/>
-    <mergeCell ref="B333:E333"/>
-    <mergeCell ref="B342:E342"/>
-    <mergeCell ref="B347:E347"/>
-    <mergeCell ref="B361:E361"/>
-    <mergeCell ref="B368:E368"/>
-    <mergeCell ref="B528:E528"/>
-    <mergeCell ref="B529:E529"/>
-    <mergeCell ref="B530:E530"/>
-    <mergeCell ref="B531:E531"/>
-    <mergeCell ref="B532:E532"/>
-    <mergeCell ref="B367:E367"/>
-    <mergeCell ref="B370:E370"/>
-    <mergeCell ref="B506:E506"/>
-    <mergeCell ref="B507:E507"/>
-    <mergeCell ref="B508:E508"/>
-    <mergeCell ref="B509:E509"/>
-    <mergeCell ref="B510:E510"/>
-    <mergeCell ref="B371:E371"/>
-    <mergeCell ref="B410:E410"/>
-    <mergeCell ref="B408:E408"/>
-    <mergeCell ref="B374:E374"/>
-    <mergeCell ref="B436:E436"/>
-    <mergeCell ref="B449:E449"/>
-    <mergeCell ref="B459:E459"/>
-    <mergeCell ref="B460:E460"/>
-    <mergeCell ref="B461:E461"/>
-    <mergeCell ref="B465:E465"/>
-    <mergeCell ref="B478:E478"/>
-    <mergeCell ref="B479:E479"/>
-    <mergeCell ref="B551:E551"/>
-    <mergeCell ref="B552:E552"/>
-    <mergeCell ref="B553:E553"/>
-    <mergeCell ref="B557:E557"/>
-    <mergeCell ref="B561:E561"/>
-    <mergeCell ref="B562:E562"/>
-    <mergeCell ref="B563:E563"/>
-    <mergeCell ref="B606:E606"/>
-    <mergeCell ref="B599:E599"/>
-    <mergeCell ref="B595:E595"/>
-    <mergeCell ref="B596:E596"/>
-    <mergeCell ref="B597:E597"/>
-    <mergeCell ref="B598:E598"/>
-    <mergeCell ref="B558:E558"/>
-    <mergeCell ref="B559:E559"/>
-    <mergeCell ref="B556:E556"/>
-    <mergeCell ref="B605:E605"/>
-    <mergeCell ref="B567:E567"/>
-    <mergeCell ref="B564:E564"/>
-    <mergeCell ref="B565:E565"/>
-    <mergeCell ref="B566:E566"/>
-    <mergeCell ref="B575:E575"/>
-    <mergeCell ref="B577:E577"/>
-    <mergeCell ref="B579:E579"/>
-    <mergeCell ref="B601:E601"/>
-    <mergeCell ref="B602:E602"/>
-    <mergeCell ref="B603:E603"/>
-    <mergeCell ref="B604:E604"/>
-    <mergeCell ref="B620:E620"/>
-    <mergeCell ref="B626:E626"/>
-    <mergeCell ref="B653:E653"/>
-    <mergeCell ref="B654:E654"/>
-    <mergeCell ref="B655:E655"/>
-    <mergeCell ref="B636:E636"/>
-    <mergeCell ref="B637:E637"/>
-    <mergeCell ref="B638:E638"/>
-    <mergeCell ref="B639:E639"/>
-    <mergeCell ref="B640:E640"/>
-    <mergeCell ref="B641:E641"/>
-    <mergeCell ref="B652:E652"/>
-    <mergeCell ref="B642:E642"/>
-    <mergeCell ref="B643:E643"/>
-    <mergeCell ref="B644:E644"/>
-    <mergeCell ref="B645:E645"/>
-    <mergeCell ref="B646:E646"/>
-    <mergeCell ref="B648:E648"/>
-    <mergeCell ref="B649:E649"/>
-    <mergeCell ref="B650:E650"/>
-    <mergeCell ref="B651:E651"/>
-    <mergeCell ref="B695:E695"/>
-    <mergeCell ref="B696:E696"/>
-    <mergeCell ref="B697:E697"/>
-    <mergeCell ref="B698:E698"/>
-    <mergeCell ref="B699:E699"/>
-    <mergeCell ref="B701:E701"/>
-    <mergeCell ref="B657:E657"/>
-    <mergeCell ref="B658:E658"/>
-    <mergeCell ref="B659:E659"/>
-    <mergeCell ref="B660:E660"/>
-    <mergeCell ref="B667:E667"/>
-    <mergeCell ref="B668:E668"/>
-    <mergeCell ref="B669:E669"/>
-    <mergeCell ref="B670:E670"/>
-    <mergeCell ref="B671:E671"/>
-    <mergeCell ref="B672:E672"/>
-    <mergeCell ref="B673:E673"/>
-    <mergeCell ref="B674:E674"/>
-    <mergeCell ref="B675:E675"/>
-    <mergeCell ref="B687:E687"/>
-    <mergeCell ref="B688:E688"/>
-    <mergeCell ref="B691:E691"/>
-    <mergeCell ref="B692:E692"/>
+    <mergeCell ref="B677:E677"/>
+    <mergeCell ref="B678:E678"/>
+    <mergeCell ref="B680:E680"/>
+    <mergeCell ref="B681:E681"/>
+    <mergeCell ref="B682:E682"/>
+    <mergeCell ref="B683:E683"/>
+    <mergeCell ref="B684:E684"/>
+    <mergeCell ref="B685:E685"/>
+    <mergeCell ref="B686:E686"/>
+    <mergeCell ref="B703:E703"/>
+    <mergeCell ref="B706:E706"/>
+    <mergeCell ref="B707:E707"/>
+    <mergeCell ref="B708:E708"/>
+    <mergeCell ref="B709:E709"/>
+    <mergeCell ref="B710:E710"/>
+    <mergeCell ref="B711:E711"/>
+    <mergeCell ref="B712:E712"/>
+    <mergeCell ref="B693:E693"/>
+    <mergeCell ref="B722:E722"/>
+    <mergeCell ref="B723:E723"/>
+    <mergeCell ref="B724:E724"/>
+    <mergeCell ref="B725:E725"/>
+    <mergeCell ref="B704:E704"/>
+    <mergeCell ref="B726:E726"/>
+    <mergeCell ref="B713:E713"/>
+    <mergeCell ref="B714:E714"/>
+    <mergeCell ref="B715:E715"/>
+    <mergeCell ref="B716:E716"/>
+    <mergeCell ref="B717:E717"/>
+    <mergeCell ref="B718:E718"/>
+    <mergeCell ref="B719:E719"/>
+    <mergeCell ref="B720:E720"/>
+    <mergeCell ref="B721:E721"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="G56" r:id="rId1" display="106" xr:uid="{91711D96-DEE6-4487-B096-595B3971FA7B}"/>

</xml_diff>

<commit_message>
Update LSP management spreadsheet
</commit_message>
<xml_diff>
--- a/data/20251229_LSP管理.xlsx
+++ b/data/20251229_LSP管理.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30215"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30219"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hiraizumitatsuya/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{84726649-ED8F-45D3-B7E3-A504ADBCFE80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{B1793B22-65D6-4830-907D-B3B2E1BB56D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="33600" windowHeight="20500" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="33600" windowHeight="20500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="マイル管理" sheetId="5" r:id="rId1"/>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2974" uniqueCount="396">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2992" uniqueCount="397">
   <si>
     <t>日付</t>
   </si>
@@ -1216,6 +1216,9 @@
     <t>JAL630</t>
   </si>
   <si>
+    <t>JAL481</t>
+  </si>
+  <si>
     <t>総額</t>
   </si>
   <si>
@@ -2403,10 +2406,10 @@
                   <c:v>2000</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>6842</c:v>
+                  <c:v>6884</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>141</c:v>
+                  <c:v>144</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -15042,7 +15045,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2A57836D-5153-486D-8B76-48FAFDDE1EA1}">
-  <dimension ref="A1:O726"/>
+  <dimension ref="A1:O733"/>
   <sheetFormatPr defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="13.7109375" customWidth="1"/>
@@ -15610,7 +15613,7 @@
       </c>
       <c r="O16">
         <f>SUMIFS(H11:H29999, B11:B29999, "*ＷＥＬＬＮＥＳＳ*")</f>
-        <v>6842</v>
+        <v>6884</v>
       </c>
     </row>
     <row r="17" spans="1:15">
@@ -15660,7 +15663,7 @@
       </c>
       <c r="O17">
         <f>SUMIFS(H11:H29999, B11:B29999, "*ＪＭＢアプリ*")</f>
-        <v>141</v>
+        <v>144</v>
       </c>
     </row>
     <row r="18" spans="1:15" ht="14.25" customHeight="1">
@@ -15852,7 +15855,7 @@
       <c r="N21" s="31"/>
       <c r="O21">
         <f>SUM(O12:O18)</f>
-        <v>168129</v>
+        <v>168174</v>
       </c>
     </row>
     <row r="22" spans="1:15">
@@ -43144,31 +43147,31 @@
       </c>
     </row>
     <row r="726" spans="1:13">
-      <c r="A726" s="29">
+      <c r="A726" s="27">
         <v>46196</v>
       </c>
-      <c r="B726" s="78" t="s">
+      <c r="B726" s="76" t="s">
         <v>33</v>
       </c>
-      <c r="C726" s="78"/>
-      <c r="D726" s="78"/>
-      <c r="E726" s="79"/>
-      <c r="F726" s="75">
-        <v>0</v>
-      </c>
-      <c r="G726" s="75">
+      <c r="C726" s="76"/>
+      <c r="D726" s="76"/>
+      <c r="E726" s="77"/>
+      <c r="F726" s="74">
+        <v>0</v>
+      </c>
+      <c r="G726" s="74">
         <v>8</v>
       </c>
-      <c r="H726" s="75">
+      <c r="H726" s="74">
         <v>8</v>
       </c>
-      <c r="I726" s="30">
+      <c r="I726" s="4">
         <v>81564</v>
       </c>
-      <c r="J726" s="75">
-        <v>0</v>
-      </c>
-      <c r="K726" s="75">
+      <c r="J726" s="74">
+        <v>0</v>
+      </c>
+      <c r="K726" s="74">
         <v>0</v>
       </c>
       <c r="L726" s="74">
@@ -43180,9 +43183,750 @@
         <v>133</v>
       </c>
     </row>
+    <row r="727" spans="1:13">
+      <c r="A727" s="27">
+        <v>46197</v>
+      </c>
+      <c r="B727" s="76" t="s">
+        <v>33</v>
+      </c>
+      <c r="C727" s="76"/>
+      <c r="D727" s="76"/>
+      <c r="E727" s="77"/>
+      <c r="F727" s="74">
+        <v>0</v>
+      </c>
+      <c r="G727" s="74">
+        <v>12</v>
+      </c>
+      <c r="H727" s="74">
+        <v>12</v>
+      </c>
+      <c r="I727" s="4">
+        <v>81576</v>
+      </c>
+      <c r="J727" s="74">
+        <v>0</v>
+      </c>
+      <c r="K727" s="74">
+        <v>0</v>
+      </c>
+      <c r="L727" s="74">
+        <f t="shared" ref="L727:L733" si="104">J727+L726</f>
+        <v>85476</v>
+      </c>
+      <c r="M727" s="74">
+        <f t="shared" ref="M727:M733" si="105">K727+M726</f>
+        <v>133</v>
+      </c>
+    </row>
+    <row r="728" spans="1:13">
+      <c r="A728" s="27">
+        <v>46198</v>
+      </c>
+      <c r="B728" s="76" t="s">
+        <v>33</v>
+      </c>
+      <c r="C728" s="76"/>
+      <c r="D728" s="76"/>
+      <c r="E728" s="77"/>
+      <c r="F728" s="74">
+        <v>0</v>
+      </c>
+      <c r="G728" s="74">
+        <v>10</v>
+      </c>
+      <c r="H728" s="74">
+        <v>10</v>
+      </c>
+      <c r="I728" s="4">
+        <v>81586</v>
+      </c>
+      <c r="J728" s="74">
+        <v>0</v>
+      </c>
+      <c r="K728" s="74">
+        <v>0</v>
+      </c>
+      <c r="L728" s="74">
+        <f t="shared" si="104"/>
+        <v>85476</v>
+      </c>
+      <c r="M728" s="74">
+        <f t="shared" si="105"/>
+        <v>133</v>
+      </c>
+    </row>
+    <row r="729" spans="1:13">
+      <c r="A729" s="27">
+        <v>46199</v>
+      </c>
+      <c r="B729" s="76" t="s">
+        <v>49</v>
+      </c>
+      <c r="C729" s="76"/>
+      <c r="D729" s="76"/>
+      <c r="E729" s="77"/>
+      <c r="F729" s="74">
+        <v>0</v>
+      </c>
+      <c r="G729" s="74">
+        <v>1</v>
+      </c>
+      <c r="H729" s="74">
+        <v>1</v>
+      </c>
+      <c r="I729" s="4">
+        <v>81587</v>
+      </c>
+      <c r="J729" s="74">
+        <v>0</v>
+      </c>
+      <c r="K729" s="74">
+        <v>0</v>
+      </c>
+      <c r="L729" s="74">
+        <f t="shared" si="104"/>
+        <v>85476</v>
+      </c>
+      <c r="M729" s="74">
+        <f t="shared" si="105"/>
+        <v>133</v>
+      </c>
+    </row>
+    <row r="730" spans="1:13">
+      <c r="A730" s="27">
+        <v>46199</v>
+      </c>
+      <c r="B730" s="76" t="s">
+        <v>33</v>
+      </c>
+      <c r="C730" s="76"/>
+      <c r="D730" s="76"/>
+      <c r="E730" s="77"/>
+      <c r="F730" s="74">
+        <v>0</v>
+      </c>
+      <c r="G730" s="74">
+        <v>11</v>
+      </c>
+      <c r="H730" s="74">
+        <v>11</v>
+      </c>
+      <c r="I730" s="4">
+        <v>81598</v>
+      </c>
+      <c r="J730" s="74">
+        <v>0</v>
+      </c>
+      <c r="K730" s="74">
+        <v>0</v>
+      </c>
+      <c r="L730" s="74">
+        <f t="shared" si="104"/>
+        <v>85476</v>
+      </c>
+      <c r="M730" s="74">
+        <f t="shared" si="105"/>
+        <v>133</v>
+      </c>
+    </row>
+    <row r="731" spans="1:13">
+      <c r="A731" s="27">
+        <v>46199</v>
+      </c>
+      <c r="B731" s="76" t="s">
+        <v>49</v>
+      </c>
+      <c r="C731" s="76"/>
+      <c r="D731" s="76"/>
+      <c r="E731" s="77"/>
+      <c r="F731" s="74">
+        <v>0</v>
+      </c>
+      <c r="G731" s="74">
+        <v>1</v>
+      </c>
+      <c r="H731" s="74">
+        <v>1</v>
+      </c>
+      <c r="I731" s="4">
+        <v>81599</v>
+      </c>
+      <c r="J731" s="74">
+        <v>0</v>
+      </c>
+      <c r="K731" s="74">
+        <v>0</v>
+      </c>
+      <c r="L731" s="74">
+        <f t="shared" si="104"/>
+        <v>85476</v>
+      </c>
+      <c r="M731" s="74">
+        <f t="shared" si="105"/>
+        <v>133</v>
+      </c>
+    </row>
+    <row r="732" spans="1:13">
+      <c r="A732" s="27">
+        <v>46199</v>
+      </c>
+      <c r="B732" s="76" t="s">
+        <v>49</v>
+      </c>
+      <c r="C732" s="76"/>
+      <c r="D732" s="76"/>
+      <c r="E732" s="77"/>
+      <c r="F732" s="74">
+        <v>0</v>
+      </c>
+      <c r="G732" s="74">
+        <v>1</v>
+      </c>
+      <c r="H732" s="74">
+        <v>1</v>
+      </c>
+      <c r="I732" s="4">
+        <v>81600</v>
+      </c>
+      <c r="J732" s="74">
+        <v>0</v>
+      </c>
+      <c r="K732" s="74">
+        <v>0</v>
+      </c>
+      <c r="L732" s="74">
+        <f t="shared" si="104"/>
+        <v>85476</v>
+      </c>
+      <c r="M732" s="74">
+        <f t="shared" si="105"/>
+        <v>133</v>
+      </c>
+    </row>
+    <row r="733" spans="1:13">
+      <c r="A733" s="29">
+        <v>46200</v>
+      </c>
+      <c r="B733" s="78" t="s">
+        <v>33</v>
+      </c>
+      <c r="C733" s="78"/>
+      <c r="D733" s="78"/>
+      <c r="E733" s="79"/>
+      <c r="F733" s="75">
+        <v>0</v>
+      </c>
+      <c r="G733" s="75">
+        <v>9</v>
+      </c>
+      <c r="H733" s="75">
+        <v>9</v>
+      </c>
+      <c r="I733" s="30">
+        <v>81609</v>
+      </c>
+      <c r="J733" s="75">
+        <v>0</v>
+      </c>
+      <c r="K733" s="75">
+        <v>0</v>
+      </c>
+      <c r="L733" s="74">
+        <f t="shared" si="104"/>
+        <v>85476</v>
+      </c>
+      <c r="M733" s="74">
+        <f t="shared" si="105"/>
+        <v>133</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:O523" xr:uid="{2A57836D-5153-486D-8B76-48FAFDDE1EA1}"/>
-  <mergeCells count="499">
+  <mergeCells count="506">
+    <mergeCell ref="B727:E727"/>
+    <mergeCell ref="B728:E728"/>
+    <mergeCell ref="B729:E729"/>
+    <mergeCell ref="B730:E730"/>
+    <mergeCell ref="B731:E731"/>
+    <mergeCell ref="B732:E732"/>
+    <mergeCell ref="B733:E733"/>
+    <mergeCell ref="B722:E722"/>
+    <mergeCell ref="B723:E723"/>
+    <mergeCell ref="B724:E724"/>
+    <mergeCell ref="B725:E725"/>
+    <mergeCell ref="B726:E726"/>
+    <mergeCell ref="B713:E713"/>
+    <mergeCell ref="B714:E714"/>
+    <mergeCell ref="B715:E715"/>
+    <mergeCell ref="B716:E716"/>
+    <mergeCell ref="B717:E717"/>
+    <mergeCell ref="B718:E718"/>
+    <mergeCell ref="B719:E719"/>
+    <mergeCell ref="B720:E720"/>
+    <mergeCell ref="B721:E721"/>
+    <mergeCell ref="B703:E703"/>
+    <mergeCell ref="B706:E706"/>
+    <mergeCell ref="B707:E707"/>
+    <mergeCell ref="B708:E708"/>
+    <mergeCell ref="B709:E709"/>
+    <mergeCell ref="B710:E710"/>
+    <mergeCell ref="B711:E711"/>
+    <mergeCell ref="B712:E712"/>
+    <mergeCell ref="B693:E693"/>
+    <mergeCell ref="B704:E704"/>
+    <mergeCell ref="B677:E677"/>
+    <mergeCell ref="B678:E678"/>
+    <mergeCell ref="B680:E680"/>
+    <mergeCell ref="B681:E681"/>
+    <mergeCell ref="B682:E682"/>
+    <mergeCell ref="B683:E683"/>
+    <mergeCell ref="B684:E684"/>
+    <mergeCell ref="B685:E685"/>
+    <mergeCell ref="B686:E686"/>
+    <mergeCell ref="B594:E594"/>
+    <mergeCell ref="B627:E627"/>
+    <mergeCell ref="B647:E647"/>
+    <mergeCell ref="B661:E661"/>
+    <mergeCell ref="B662:E662"/>
+    <mergeCell ref="B663:E663"/>
+    <mergeCell ref="B664:E664"/>
+    <mergeCell ref="B665:E665"/>
+    <mergeCell ref="B666:E666"/>
+    <mergeCell ref="B633:E633"/>
+    <mergeCell ref="B634:E634"/>
+    <mergeCell ref="B635:E635"/>
+    <mergeCell ref="B611:E611"/>
+    <mergeCell ref="B628:E628"/>
+    <mergeCell ref="B629:E629"/>
+    <mergeCell ref="B630:E630"/>
+    <mergeCell ref="B631:E631"/>
+    <mergeCell ref="B632:E632"/>
+    <mergeCell ref="B621:E621"/>
+    <mergeCell ref="B622:E622"/>
+    <mergeCell ref="B623:E623"/>
+    <mergeCell ref="B624:E624"/>
+    <mergeCell ref="B625:E625"/>
+    <mergeCell ref="B600:E600"/>
+    <mergeCell ref="B569:E569"/>
+    <mergeCell ref="B570:E570"/>
+    <mergeCell ref="B571:E571"/>
+    <mergeCell ref="B572:E572"/>
+    <mergeCell ref="B573:E573"/>
+    <mergeCell ref="B576:E576"/>
+    <mergeCell ref="B578:E578"/>
+    <mergeCell ref="B591:E591"/>
+    <mergeCell ref="B592:E592"/>
+    <mergeCell ref="B580:E580"/>
+    <mergeCell ref="B589:E589"/>
+    <mergeCell ref="B511:E511"/>
+    <mergeCell ref="B512:E512"/>
+    <mergeCell ref="B513:E513"/>
+    <mergeCell ref="B514:E514"/>
+    <mergeCell ref="B515:E515"/>
+    <mergeCell ref="B535:E535"/>
+    <mergeCell ref="B537:E537"/>
+    <mergeCell ref="B555:E555"/>
+    <mergeCell ref="B560:E560"/>
+    <mergeCell ref="B548:E548"/>
+    <mergeCell ref="B549:E549"/>
+    <mergeCell ref="B546:E546"/>
+    <mergeCell ref="B547:E547"/>
+    <mergeCell ref="B533:E533"/>
+    <mergeCell ref="B534:E534"/>
+    <mergeCell ref="B536:E536"/>
+    <mergeCell ref="B538:E538"/>
+    <mergeCell ref="B539:E539"/>
+    <mergeCell ref="B540:E540"/>
+    <mergeCell ref="B541:E541"/>
+    <mergeCell ref="B543:E543"/>
+    <mergeCell ref="B544:E544"/>
+    <mergeCell ref="B526:E526"/>
+    <mergeCell ref="B527:E527"/>
+    <mergeCell ref="B505:E505"/>
+    <mergeCell ref="B480:E480"/>
+    <mergeCell ref="B469:E469"/>
+    <mergeCell ref="B481:E481"/>
+    <mergeCell ref="B490:E490"/>
+    <mergeCell ref="B491:E491"/>
+    <mergeCell ref="B492:E492"/>
+    <mergeCell ref="B493:E493"/>
+    <mergeCell ref="B494:E494"/>
+    <mergeCell ref="B498:E498"/>
+    <mergeCell ref="B499:E499"/>
+    <mergeCell ref="B500:E500"/>
+    <mergeCell ref="B501:E501"/>
+    <mergeCell ref="B502:E502"/>
+    <mergeCell ref="B503:E503"/>
+    <mergeCell ref="B504:E504"/>
+    <mergeCell ref="B482:E482"/>
+    <mergeCell ref="B495:E495"/>
+    <mergeCell ref="B377:E377"/>
+    <mergeCell ref="B378:E378"/>
+    <mergeCell ref="B379:E379"/>
+    <mergeCell ref="B388:E388"/>
+    <mergeCell ref="B395:E395"/>
+    <mergeCell ref="B400:E400"/>
+    <mergeCell ref="B402:E402"/>
+    <mergeCell ref="B393:E393"/>
+    <mergeCell ref="B396:E396"/>
+    <mergeCell ref="B398:E398"/>
+    <mergeCell ref="B399:E399"/>
+    <mergeCell ref="B401:E401"/>
+    <mergeCell ref="B386:E386"/>
+    <mergeCell ref="B292:E292"/>
+    <mergeCell ref="B458:E458"/>
+    <mergeCell ref="B466:E466"/>
+    <mergeCell ref="B467:E467"/>
+    <mergeCell ref="B468:E468"/>
+    <mergeCell ref="B426:E426"/>
+    <mergeCell ref="B438:E438"/>
+    <mergeCell ref="B439:E439"/>
+    <mergeCell ref="B453:E453"/>
+    <mergeCell ref="B454:E454"/>
+    <mergeCell ref="B455:E455"/>
+    <mergeCell ref="B456:E456"/>
+    <mergeCell ref="B457:E457"/>
+    <mergeCell ref="B442:E442"/>
+    <mergeCell ref="B450:E450"/>
+    <mergeCell ref="B451:E451"/>
+    <mergeCell ref="B387:E387"/>
+    <mergeCell ref="B389:E389"/>
+    <mergeCell ref="B390:E390"/>
+    <mergeCell ref="B392:E392"/>
+    <mergeCell ref="B403:E403"/>
+    <mergeCell ref="B404:E404"/>
+    <mergeCell ref="B406:E406"/>
+    <mergeCell ref="B409:E409"/>
+    <mergeCell ref="B259:E259"/>
+    <mergeCell ref="B412:E412"/>
+    <mergeCell ref="B419:E419"/>
+    <mergeCell ref="B425:E425"/>
+    <mergeCell ref="B452:E452"/>
+    <mergeCell ref="B262:E262"/>
+    <mergeCell ref="B264:E264"/>
+    <mergeCell ref="B266:E266"/>
+    <mergeCell ref="B276:E276"/>
+    <mergeCell ref="B277:E277"/>
+    <mergeCell ref="B278:E278"/>
+    <mergeCell ref="B279:E279"/>
+    <mergeCell ref="B280:E280"/>
+    <mergeCell ref="B281:E281"/>
+    <mergeCell ref="B282:E282"/>
+    <mergeCell ref="B283:E283"/>
+    <mergeCell ref="B284:E284"/>
+    <mergeCell ref="B285:E285"/>
+    <mergeCell ref="B286:E286"/>
+    <mergeCell ref="B287:E287"/>
+    <mergeCell ref="B288:E288"/>
+    <mergeCell ref="B289:E289"/>
+    <mergeCell ref="B290:E290"/>
+    <mergeCell ref="B291:E291"/>
+    <mergeCell ref="B260:E260"/>
+    <mergeCell ref="B261:E261"/>
+    <mergeCell ref="B241:E241"/>
+    <mergeCell ref="B242:E242"/>
+    <mergeCell ref="B245:E245"/>
+    <mergeCell ref="B247:E247"/>
+    <mergeCell ref="B248:E248"/>
+    <mergeCell ref="B229:E229"/>
+    <mergeCell ref="B230:E230"/>
+    <mergeCell ref="B231:E231"/>
+    <mergeCell ref="B232:E232"/>
+    <mergeCell ref="B233:E233"/>
+    <mergeCell ref="B234:E234"/>
+    <mergeCell ref="B235:E235"/>
+    <mergeCell ref="B236:E236"/>
+    <mergeCell ref="B237:E237"/>
+    <mergeCell ref="B238:E238"/>
+    <mergeCell ref="B239:E239"/>
+    <mergeCell ref="B240:E240"/>
+    <mergeCell ref="B250:E250"/>
+    <mergeCell ref="B251:E251"/>
+    <mergeCell ref="B253:E253"/>
+    <mergeCell ref="B255:E255"/>
+    <mergeCell ref="B257:E257"/>
+    <mergeCell ref="B226:E226"/>
+    <mergeCell ref="B227:E227"/>
+    <mergeCell ref="B228:E228"/>
+    <mergeCell ref="B218:E218"/>
+    <mergeCell ref="B219:E219"/>
+    <mergeCell ref="B220:E220"/>
+    <mergeCell ref="B221:E221"/>
+    <mergeCell ref="B222:E222"/>
+    <mergeCell ref="B223:E223"/>
+    <mergeCell ref="B198:E198"/>
+    <mergeCell ref="B201:E201"/>
+    <mergeCell ref="B202:E202"/>
+    <mergeCell ref="B203:E203"/>
+    <mergeCell ref="B204:E204"/>
+    <mergeCell ref="B205:E205"/>
+    <mergeCell ref="B206:E206"/>
+    <mergeCell ref="B224:E224"/>
+    <mergeCell ref="B225:E225"/>
+    <mergeCell ref="B102:E102"/>
+    <mergeCell ref="B94:E94"/>
+    <mergeCell ref="B95:E95"/>
+    <mergeCell ref="B96:E96"/>
+    <mergeCell ref="B98:E98"/>
+    <mergeCell ref="B100:E100"/>
+    <mergeCell ref="B89:E89"/>
+    <mergeCell ref="B90:E90"/>
+    <mergeCell ref="B91:E91"/>
+    <mergeCell ref="B92:E92"/>
+    <mergeCell ref="B93:E93"/>
+    <mergeCell ref="B103:E103"/>
+    <mergeCell ref="B84:E84"/>
+    <mergeCell ref="B85:E85"/>
+    <mergeCell ref="B86:E86"/>
+    <mergeCell ref="B87:E87"/>
+    <mergeCell ref="B88:E88"/>
+    <mergeCell ref="B10:E10"/>
+    <mergeCell ref="B35:E35"/>
+    <mergeCell ref="B36:E36"/>
+    <mergeCell ref="B37:E37"/>
+    <mergeCell ref="B53:E53"/>
+    <mergeCell ref="B61:E61"/>
+    <mergeCell ref="B62:E62"/>
+    <mergeCell ref="B63:E63"/>
+    <mergeCell ref="B65:E65"/>
+    <mergeCell ref="B54:E54"/>
+    <mergeCell ref="B55:E55"/>
+    <mergeCell ref="B57:E57"/>
+    <mergeCell ref="B58:E58"/>
+    <mergeCell ref="B59:E59"/>
+    <mergeCell ref="B81:E81"/>
+    <mergeCell ref="B82:E82"/>
+    <mergeCell ref="B83:E83"/>
+    <mergeCell ref="B101:E101"/>
+    <mergeCell ref="B78:E78"/>
+    <mergeCell ref="B40:E40"/>
+    <mergeCell ref="B41:E41"/>
+    <mergeCell ref="B42:E42"/>
+    <mergeCell ref="B43:E43"/>
+    <mergeCell ref="B44:E44"/>
+    <mergeCell ref="B29:E29"/>
+    <mergeCell ref="B30:E30"/>
+    <mergeCell ref="B31:E31"/>
+    <mergeCell ref="B32:E32"/>
+    <mergeCell ref="B33:E33"/>
+    <mergeCell ref="B34:E34"/>
+    <mergeCell ref="B60:E60"/>
+    <mergeCell ref="B38:E38"/>
+    <mergeCell ref="B49:E49"/>
+    <mergeCell ref="B50:E50"/>
+    <mergeCell ref="B51:E51"/>
+    <mergeCell ref="B52:E52"/>
+    <mergeCell ref="B47:E47"/>
+    <mergeCell ref="B48:E48"/>
+    <mergeCell ref="B45:E45"/>
+    <mergeCell ref="B46:E46"/>
+    <mergeCell ref="B39:E39"/>
+    <mergeCell ref="B71:E71"/>
+    <mergeCell ref="B72:E72"/>
+    <mergeCell ref="B74:E74"/>
+    <mergeCell ref="B76:E76"/>
+    <mergeCell ref="B77:E77"/>
+    <mergeCell ref="B66:E66"/>
+    <mergeCell ref="B67:E67"/>
+    <mergeCell ref="B68:E68"/>
+    <mergeCell ref="B69:E69"/>
+    <mergeCell ref="B70:E70"/>
+    <mergeCell ref="B104:E104"/>
+    <mergeCell ref="B105:E105"/>
+    <mergeCell ref="B106:E106"/>
+    <mergeCell ref="B107:E107"/>
+    <mergeCell ref="B108:E108"/>
+    <mergeCell ref="B109:E109"/>
+    <mergeCell ref="B110:E110"/>
+    <mergeCell ref="B111:E111"/>
+    <mergeCell ref="B145:E145"/>
+    <mergeCell ref="B135:E135"/>
+    <mergeCell ref="B122:E122"/>
+    <mergeCell ref="B123:E123"/>
+    <mergeCell ref="B124:E124"/>
+    <mergeCell ref="B125:E125"/>
+    <mergeCell ref="B126:E126"/>
+    <mergeCell ref="B146:E146"/>
+    <mergeCell ref="B112:E112"/>
+    <mergeCell ref="B120:E120"/>
+    <mergeCell ref="B121:E121"/>
+    <mergeCell ref="B114:E114"/>
+    <mergeCell ref="B115:E115"/>
+    <mergeCell ref="B117:E117"/>
+    <mergeCell ref="B118:E118"/>
+    <mergeCell ref="B119:E119"/>
+    <mergeCell ref="B127:E127"/>
+    <mergeCell ref="B142:E142"/>
+    <mergeCell ref="B143:E143"/>
+    <mergeCell ref="B144:E144"/>
+    <mergeCell ref="B137:E137"/>
+    <mergeCell ref="B138:E138"/>
+    <mergeCell ref="B139:E139"/>
+    <mergeCell ref="B140:E140"/>
+    <mergeCell ref="B141:E141"/>
+    <mergeCell ref="B128:E128"/>
+    <mergeCell ref="B129:E129"/>
+    <mergeCell ref="B130:E130"/>
+    <mergeCell ref="B131:E131"/>
+    <mergeCell ref="B132:E132"/>
+    <mergeCell ref="B134:E134"/>
+    <mergeCell ref="B147:E147"/>
+    <mergeCell ref="B148:E148"/>
+    <mergeCell ref="B149:E149"/>
+    <mergeCell ref="B157:E157"/>
+    <mergeCell ref="B167:E167"/>
+    <mergeCell ref="B168:E168"/>
+    <mergeCell ref="B169:E169"/>
+    <mergeCell ref="B170:E170"/>
+    <mergeCell ref="B171:E171"/>
+    <mergeCell ref="B172:E172"/>
+    <mergeCell ref="B174:E174"/>
+    <mergeCell ref="B175:E175"/>
+    <mergeCell ref="B176:E176"/>
+    <mergeCell ref="B178:E178"/>
+    <mergeCell ref="B179:E179"/>
+    <mergeCell ref="B187:E187"/>
+    <mergeCell ref="B188:E188"/>
+    <mergeCell ref="B217:E217"/>
+    <mergeCell ref="B207:E207"/>
+    <mergeCell ref="B209:E209"/>
+    <mergeCell ref="B210:E210"/>
+    <mergeCell ref="B212:E212"/>
+    <mergeCell ref="B214:E214"/>
+    <mergeCell ref="B215:E215"/>
+    <mergeCell ref="B216:E216"/>
+    <mergeCell ref="B189:E189"/>
+    <mergeCell ref="B190:E190"/>
+    <mergeCell ref="B191:E191"/>
+    <mergeCell ref="B193:E193"/>
+    <mergeCell ref="B194:E194"/>
+    <mergeCell ref="B195:E195"/>
+    <mergeCell ref="B196:E196"/>
+    <mergeCell ref="B197:E197"/>
+    <mergeCell ref="B293:E293"/>
+    <mergeCell ref="B294:E294"/>
+    <mergeCell ref="B295:E295"/>
+    <mergeCell ref="B296:E296"/>
+    <mergeCell ref="B297:E297"/>
+    <mergeCell ref="B299:E299"/>
+    <mergeCell ref="B300:E300"/>
+    <mergeCell ref="B301:E301"/>
+    <mergeCell ref="B302:E302"/>
+    <mergeCell ref="B369:E369"/>
+    <mergeCell ref="B320:E320"/>
+    <mergeCell ref="B321:E321"/>
+    <mergeCell ref="B322:E322"/>
+    <mergeCell ref="B323:E323"/>
+    <mergeCell ref="B324:E324"/>
+    <mergeCell ref="B360:E360"/>
+    <mergeCell ref="B362:E362"/>
+    <mergeCell ref="B364:E364"/>
+    <mergeCell ref="B365:E365"/>
+    <mergeCell ref="B327:E327"/>
+    <mergeCell ref="B328:E328"/>
+    <mergeCell ref="B332:E332"/>
+    <mergeCell ref="B356:E356"/>
+    <mergeCell ref="B357:E357"/>
+    <mergeCell ref="B358:E358"/>
+    <mergeCell ref="B359:E359"/>
+    <mergeCell ref="B375:E375"/>
+    <mergeCell ref="B376:E376"/>
+    <mergeCell ref="B319:E319"/>
+    <mergeCell ref="B303:E303"/>
+    <mergeCell ref="B304:E304"/>
+    <mergeCell ref="B306:E306"/>
+    <mergeCell ref="B307:E307"/>
+    <mergeCell ref="B308:E308"/>
+    <mergeCell ref="B309:E309"/>
+    <mergeCell ref="B311:E311"/>
+    <mergeCell ref="B312:E312"/>
+    <mergeCell ref="B313:E313"/>
+    <mergeCell ref="B314:E314"/>
+    <mergeCell ref="B315:E315"/>
+    <mergeCell ref="B316:E316"/>
+    <mergeCell ref="B317:E317"/>
+    <mergeCell ref="B318:E318"/>
+    <mergeCell ref="B325:E325"/>
+    <mergeCell ref="B329:E329"/>
+    <mergeCell ref="B333:E333"/>
+    <mergeCell ref="B342:E342"/>
+    <mergeCell ref="B347:E347"/>
+    <mergeCell ref="B361:E361"/>
+    <mergeCell ref="B368:E368"/>
+    <mergeCell ref="B528:E528"/>
+    <mergeCell ref="B529:E529"/>
+    <mergeCell ref="B530:E530"/>
+    <mergeCell ref="B531:E531"/>
+    <mergeCell ref="B532:E532"/>
+    <mergeCell ref="B367:E367"/>
+    <mergeCell ref="B370:E370"/>
+    <mergeCell ref="B506:E506"/>
+    <mergeCell ref="B507:E507"/>
+    <mergeCell ref="B508:E508"/>
+    <mergeCell ref="B509:E509"/>
+    <mergeCell ref="B510:E510"/>
+    <mergeCell ref="B371:E371"/>
+    <mergeCell ref="B410:E410"/>
+    <mergeCell ref="B408:E408"/>
+    <mergeCell ref="B374:E374"/>
+    <mergeCell ref="B436:E436"/>
+    <mergeCell ref="B449:E449"/>
+    <mergeCell ref="B459:E459"/>
+    <mergeCell ref="B460:E460"/>
+    <mergeCell ref="B461:E461"/>
+    <mergeCell ref="B465:E465"/>
+    <mergeCell ref="B478:E478"/>
+    <mergeCell ref="B479:E479"/>
+    <mergeCell ref="B551:E551"/>
+    <mergeCell ref="B552:E552"/>
+    <mergeCell ref="B553:E553"/>
+    <mergeCell ref="B557:E557"/>
+    <mergeCell ref="B561:E561"/>
+    <mergeCell ref="B562:E562"/>
+    <mergeCell ref="B563:E563"/>
+    <mergeCell ref="B606:E606"/>
+    <mergeCell ref="B599:E599"/>
+    <mergeCell ref="B595:E595"/>
+    <mergeCell ref="B596:E596"/>
+    <mergeCell ref="B597:E597"/>
+    <mergeCell ref="B598:E598"/>
+    <mergeCell ref="B558:E558"/>
+    <mergeCell ref="B559:E559"/>
+    <mergeCell ref="B556:E556"/>
+    <mergeCell ref="B605:E605"/>
+    <mergeCell ref="B567:E567"/>
+    <mergeCell ref="B564:E564"/>
+    <mergeCell ref="B565:E565"/>
+    <mergeCell ref="B566:E566"/>
+    <mergeCell ref="B575:E575"/>
+    <mergeCell ref="B577:E577"/>
+    <mergeCell ref="B579:E579"/>
+    <mergeCell ref="B601:E601"/>
+    <mergeCell ref="B602:E602"/>
+    <mergeCell ref="B603:E603"/>
+    <mergeCell ref="B604:E604"/>
+    <mergeCell ref="B620:E620"/>
+    <mergeCell ref="B626:E626"/>
+    <mergeCell ref="B653:E653"/>
+    <mergeCell ref="B654:E654"/>
+    <mergeCell ref="B655:E655"/>
+    <mergeCell ref="B636:E636"/>
+    <mergeCell ref="B637:E637"/>
+    <mergeCell ref="B638:E638"/>
+    <mergeCell ref="B639:E639"/>
+    <mergeCell ref="B640:E640"/>
+    <mergeCell ref="B641:E641"/>
+    <mergeCell ref="B652:E652"/>
+    <mergeCell ref="B642:E642"/>
+    <mergeCell ref="B643:E643"/>
+    <mergeCell ref="B644:E644"/>
+    <mergeCell ref="B645:E645"/>
+    <mergeCell ref="B646:E646"/>
+    <mergeCell ref="B648:E648"/>
+    <mergeCell ref="B649:E649"/>
+    <mergeCell ref="B650:E650"/>
     <mergeCell ref="B651:E651"/>
     <mergeCell ref="B695:E695"/>
     <mergeCell ref="B696:E696"/>
@@ -43207,481 +43951,6 @@
     <mergeCell ref="B688:E688"/>
     <mergeCell ref="B691:E691"/>
     <mergeCell ref="B692:E692"/>
-    <mergeCell ref="B601:E601"/>
-    <mergeCell ref="B602:E602"/>
-    <mergeCell ref="B603:E603"/>
-    <mergeCell ref="B604:E604"/>
-    <mergeCell ref="B620:E620"/>
-    <mergeCell ref="B626:E626"/>
-    <mergeCell ref="B653:E653"/>
-    <mergeCell ref="B654:E654"/>
-    <mergeCell ref="B655:E655"/>
-    <mergeCell ref="B636:E636"/>
-    <mergeCell ref="B637:E637"/>
-    <mergeCell ref="B638:E638"/>
-    <mergeCell ref="B639:E639"/>
-    <mergeCell ref="B640:E640"/>
-    <mergeCell ref="B641:E641"/>
-    <mergeCell ref="B652:E652"/>
-    <mergeCell ref="B642:E642"/>
-    <mergeCell ref="B643:E643"/>
-    <mergeCell ref="B644:E644"/>
-    <mergeCell ref="B645:E645"/>
-    <mergeCell ref="B646:E646"/>
-    <mergeCell ref="B648:E648"/>
-    <mergeCell ref="B649:E649"/>
-    <mergeCell ref="B650:E650"/>
-    <mergeCell ref="B551:E551"/>
-    <mergeCell ref="B552:E552"/>
-    <mergeCell ref="B553:E553"/>
-    <mergeCell ref="B557:E557"/>
-    <mergeCell ref="B561:E561"/>
-    <mergeCell ref="B562:E562"/>
-    <mergeCell ref="B563:E563"/>
-    <mergeCell ref="B606:E606"/>
-    <mergeCell ref="B599:E599"/>
-    <mergeCell ref="B595:E595"/>
-    <mergeCell ref="B596:E596"/>
-    <mergeCell ref="B597:E597"/>
-    <mergeCell ref="B598:E598"/>
-    <mergeCell ref="B558:E558"/>
-    <mergeCell ref="B559:E559"/>
-    <mergeCell ref="B556:E556"/>
-    <mergeCell ref="B605:E605"/>
-    <mergeCell ref="B567:E567"/>
-    <mergeCell ref="B564:E564"/>
-    <mergeCell ref="B565:E565"/>
-    <mergeCell ref="B566:E566"/>
-    <mergeCell ref="B575:E575"/>
-    <mergeCell ref="B577:E577"/>
-    <mergeCell ref="B579:E579"/>
-    <mergeCell ref="B528:E528"/>
-    <mergeCell ref="B529:E529"/>
-    <mergeCell ref="B530:E530"/>
-    <mergeCell ref="B531:E531"/>
-    <mergeCell ref="B532:E532"/>
-    <mergeCell ref="B367:E367"/>
-    <mergeCell ref="B370:E370"/>
-    <mergeCell ref="B506:E506"/>
-    <mergeCell ref="B507:E507"/>
-    <mergeCell ref="B508:E508"/>
-    <mergeCell ref="B509:E509"/>
-    <mergeCell ref="B510:E510"/>
-    <mergeCell ref="B371:E371"/>
-    <mergeCell ref="B410:E410"/>
-    <mergeCell ref="B408:E408"/>
-    <mergeCell ref="B374:E374"/>
-    <mergeCell ref="B436:E436"/>
-    <mergeCell ref="B449:E449"/>
-    <mergeCell ref="B459:E459"/>
-    <mergeCell ref="B460:E460"/>
-    <mergeCell ref="B461:E461"/>
-    <mergeCell ref="B465:E465"/>
-    <mergeCell ref="B478:E478"/>
-    <mergeCell ref="B479:E479"/>
-    <mergeCell ref="B375:E375"/>
-    <mergeCell ref="B376:E376"/>
-    <mergeCell ref="B319:E319"/>
-    <mergeCell ref="B303:E303"/>
-    <mergeCell ref="B304:E304"/>
-    <mergeCell ref="B306:E306"/>
-    <mergeCell ref="B307:E307"/>
-    <mergeCell ref="B308:E308"/>
-    <mergeCell ref="B309:E309"/>
-    <mergeCell ref="B311:E311"/>
-    <mergeCell ref="B312:E312"/>
-    <mergeCell ref="B313:E313"/>
-    <mergeCell ref="B314:E314"/>
-    <mergeCell ref="B315:E315"/>
-    <mergeCell ref="B316:E316"/>
-    <mergeCell ref="B317:E317"/>
-    <mergeCell ref="B318:E318"/>
-    <mergeCell ref="B325:E325"/>
-    <mergeCell ref="B329:E329"/>
-    <mergeCell ref="B333:E333"/>
-    <mergeCell ref="B342:E342"/>
-    <mergeCell ref="B347:E347"/>
-    <mergeCell ref="B361:E361"/>
-    <mergeCell ref="B368:E368"/>
-    <mergeCell ref="B369:E369"/>
-    <mergeCell ref="B320:E320"/>
-    <mergeCell ref="B321:E321"/>
-    <mergeCell ref="B322:E322"/>
-    <mergeCell ref="B323:E323"/>
-    <mergeCell ref="B324:E324"/>
-    <mergeCell ref="B360:E360"/>
-    <mergeCell ref="B362:E362"/>
-    <mergeCell ref="B364:E364"/>
-    <mergeCell ref="B365:E365"/>
-    <mergeCell ref="B327:E327"/>
-    <mergeCell ref="B328:E328"/>
-    <mergeCell ref="B332:E332"/>
-    <mergeCell ref="B356:E356"/>
-    <mergeCell ref="B357:E357"/>
-    <mergeCell ref="B358:E358"/>
-    <mergeCell ref="B359:E359"/>
-    <mergeCell ref="B293:E293"/>
-    <mergeCell ref="B294:E294"/>
-    <mergeCell ref="B295:E295"/>
-    <mergeCell ref="B296:E296"/>
-    <mergeCell ref="B297:E297"/>
-    <mergeCell ref="B299:E299"/>
-    <mergeCell ref="B300:E300"/>
-    <mergeCell ref="B301:E301"/>
-    <mergeCell ref="B302:E302"/>
-    <mergeCell ref="B172:E172"/>
-    <mergeCell ref="B174:E174"/>
-    <mergeCell ref="B175:E175"/>
-    <mergeCell ref="B176:E176"/>
-    <mergeCell ref="B178:E178"/>
-    <mergeCell ref="B179:E179"/>
-    <mergeCell ref="B187:E187"/>
-    <mergeCell ref="B188:E188"/>
-    <mergeCell ref="B217:E217"/>
-    <mergeCell ref="B207:E207"/>
-    <mergeCell ref="B209:E209"/>
-    <mergeCell ref="B210:E210"/>
-    <mergeCell ref="B212:E212"/>
-    <mergeCell ref="B214:E214"/>
-    <mergeCell ref="B215:E215"/>
-    <mergeCell ref="B216:E216"/>
-    <mergeCell ref="B189:E189"/>
-    <mergeCell ref="B190:E190"/>
-    <mergeCell ref="B191:E191"/>
-    <mergeCell ref="B193:E193"/>
-    <mergeCell ref="B194:E194"/>
-    <mergeCell ref="B195:E195"/>
-    <mergeCell ref="B196:E196"/>
-    <mergeCell ref="B197:E197"/>
-    <mergeCell ref="B147:E147"/>
-    <mergeCell ref="B148:E148"/>
-    <mergeCell ref="B149:E149"/>
-    <mergeCell ref="B157:E157"/>
-    <mergeCell ref="B167:E167"/>
-    <mergeCell ref="B168:E168"/>
-    <mergeCell ref="B169:E169"/>
-    <mergeCell ref="B170:E170"/>
-    <mergeCell ref="B171:E171"/>
-    <mergeCell ref="B146:E146"/>
-    <mergeCell ref="B112:E112"/>
-    <mergeCell ref="B120:E120"/>
-    <mergeCell ref="B121:E121"/>
-    <mergeCell ref="B114:E114"/>
-    <mergeCell ref="B115:E115"/>
-    <mergeCell ref="B117:E117"/>
-    <mergeCell ref="B118:E118"/>
-    <mergeCell ref="B119:E119"/>
-    <mergeCell ref="B127:E127"/>
-    <mergeCell ref="B142:E142"/>
-    <mergeCell ref="B143:E143"/>
-    <mergeCell ref="B144:E144"/>
-    <mergeCell ref="B137:E137"/>
-    <mergeCell ref="B138:E138"/>
-    <mergeCell ref="B139:E139"/>
-    <mergeCell ref="B140:E140"/>
-    <mergeCell ref="B141:E141"/>
-    <mergeCell ref="B128:E128"/>
-    <mergeCell ref="B129:E129"/>
-    <mergeCell ref="B130:E130"/>
-    <mergeCell ref="B131:E131"/>
-    <mergeCell ref="B132:E132"/>
-    <mergeCell ref="B134:E134"/>
-    <mergeCell ref="B104:E104"/>
-    <mergeCell ref="B105:E105"/>
-    <mergeCell ref="B106:E106"/>
-    <mergeCell ref="B107:E107"/>
-    <mergeCell ref="B108:E108"/>
-    <mergeCell ref="B109:E109"/>
-    <mergeCell ref="B110:E110"/>
-    <mergeCell ref="B111:E111"/>
-    <mergeCell ref="B145:E145"/>
-    <mergeCell ref="B135:E135"/>
-    <mergeCell ref="B122:E122"/>
-    <mergeCell ref="B123:E123"/>
-    <mergeCell ref="B124:E124"/>
-    <mergeCell ref="B125:E125"/>
-    <mergeCell ref="B126:E126"/>
-    <mergeCell ref="B72:E72"/>
-    <mergeCell ref="B74:E74"/>
-    <mergeCell ref="B76:E76"/>
-    <mergeCell ref="B77:E77"/>
-    <mergeCell ref="B66:E66"/>
-    <mergeCell ref="B67:E67"/>
-    <mergeCell ref="B68:E68"/>
-    <mergeCell ref="B69:E69"/>
-    <mergeCell ref="B70:E70"/>
-    <mergeCell ref="B78:E78"/>
-    <mergeCell ref="B40:E40"/>
-    <mergeCell ref="B41:E41"/>
-    <mergeCell ref="B42:E42"/>
-    <mergeCell ref="B43:E43"/>
-    <mergeCell ref="B44:E44"/>
-    <mergeCell ref="B29:E29"/>
-    <mergeCell ref="B30:E30"/>
-    <mergeCell ref="B31:E31"/>
-    <mergeCell ref="B32:E32"/>
-    <mergeCell ref="B33:E33"/>
-    <mergeCell ref="B34:E34"/>
-    <mergeCell ref="B60:E60"/>
-    <mergeCell ref="B38:E38"/>
-    <mergeCell ref="B49:E49"/>
-    <mergeCell ref="B50:E50"/>
-    <mergeCell ref="B51:E51"/>
-    <mergeCell ref="B52:E52"/>
-    <mergeCell ref="B47:E47"/>
-    <mergeCell ref="B48:E48"/>
-    <mergeCell ref="B45:E45"/>
-    <mergeCell ref="B46:E46"/>
-    <mergeCell ref="B39:E39"/>
-    <mergeCell ref="B71:E71"/>
-    <mergeCell ref="B103:E103"/>
-    <mergeCell ref="B84:E84"/>
-    <mergeCell ref="B85:E85"/>
-    <mergeCell ref="B86:E86"/>
-    <mergeCell ref="B87:E87"/>
-    <mergeCell ref="B88:E88"/>
-    <mergeCell ref="B10:E10"/>
-    <mergeCell ref="B35:E35"/>
-    <mergeCell ref="B36:E36"/>
-    <mergeCell ref="B37:E37"/>
-    <mergeCell ref="B53:E53"/>
-    <mergeCell ref="B61:E61"/>
-    <mergeCell ref="B62:E62"/>
-    <mergeCell ref="B63:E63"/>
-    <mergeCell ref="B65:E65"/>
-    <mergeCell ref="B54:E54"/>
-    <mergeCell ref="B55:E55"/>
-    <mergeCell ref="B57:E57"/>
-    <mergeCell ref="B58:E58"/>
-    <mergeCell ref="B59:E59"/>
-    <mergeCell ref="B81:E81"/>
-    <mergeCell ref="B82:E82"/>
-    <mergeCell ref="B83:E83"/>
-    <mergeCell ref="B101:E101"/>
-    <mergeCell ref="B102:E102"/>
-    <mergeCell ref="B94:E94"/>
-    <mergeCell ref="B95:E95"/>
-    <mergeCell ref="B96:E96"/>
-    <mergeCell ref="B98:E98"/>
-    <mergeCell ref="B100:E100"/>
-    <mergeCell ref="B89:E89"/>
-    <mergeCell ref="B90:E90"/>
-    <mergeCell ref="B91:E91"/>
-    <mergeCell ref="B92:E92"/>
-    <mergeCell ref="B93:E93"/>
-    <mergeCell ref="B198:E198"/>
-    <mergeCell ref="B201:E201"/>
-    <mergeCell ref="B202:E202"/>
-    <mergeCell ref="B203:E203"/>
-    <mergeCell ref="B204:E204"/>
-    <mergeCell ref="B205:E205"/>
-    <mergeCell ref="B206:E206"/>
-    <mergeCell ref="B224:E224"/>
-    <mergeCell ref="B225:E225"/>
-    <mergeCell ref="B226:E226"/>
-    <mergeCell ref="B227:E227"/>
-    <mergeCell ref="B228:E228"/>
-    <mergeCell ref="B218:E218"/>
-    <mergeCell ref="B219:E219"/>
-    <mergeCell ref="B220:E220"/>
-    <mergeCell ref="B221:E221"/>
-    <mergeCell ref="B222:E222"/>
-    <mergeCell ref="B223:E223"/>
-    <mergeCell ref="B260:E260"/>
-    <mergeCell ref="B261:E261"/>
-    <mergeCell ref="B241:E241"/>
-    <mergeCell ref="B242:E242"/>
-    <mergeCell ref="B245:E245"/>
-    <mergeCell ref="B247:E247"/>
-    <mergeCell ref="B248:E248"/>
-    <mergeCell ref="B229:E229"/>
-    <mergeCell ref="B230:E230"/>
-    <mergeCell ref="B231:E231"/>
-    <mergeCell ref="B232:E232"/>
-    <mergeCell ref="B233:E233"/>
-    <mergeCell ref="B234:E234"/>
-    <mergeCell ref="B235:E235"/>
-    <mergeCell ref="B236:E236"/>
-    <mergeCell ref="B237:E237"/>
-    <mergeCell ref="B238:E238"/>
-    <mergeCell ref="B239:E239"/>
-    <mergeCell ref="B240:E240"/>
-    <mergeCell ref="B250:E250"/>
-    <mergeCell ref="B251:E251"/>
-    <mergeCell ref="B253:E253"/>
-    <mergeCell ref="B255:E255"/>
-    <mergeCell ref="B257:E257"/>
-    <mergeCell ref="B259:E259"/>
-    <mergeCell ref="B412:E412"/>
-    <mergeCell ref="B419:E419"/>
-    <mergeCell ref="B425:E425"/>
-    <mergeCell ref="B452:E452"/>
-    <mergeCell ref="B262:E262"/>
-    <mergeCell ref="B264:E264"/>
-    <mergeCell ref="B266:E266"/>
-    <mergeCell ref="B276:E276"/>
-    <mergeCell ref="B277:E277"/>
-    <mergeCell ref="B278:E278"/>
-    <mergeCell ref="B279:E279"/>
-    <mergeCell ref="B280:E280"/>
-    <mergeCell ref="B281:E281"/>
-    <mergeCell ref="B282:E282"/>
-    <mergeCell ref="B283:E283"/>
-    <mergeCell ref="B284:E284"/>
-    <mergeCell ref="B285:E285"/>
-    <mergeCell ref="B286:E286"/>
-    <mergeCell ref="B287:E287"/>
-    <mergeCell ref="B288:E288"/>
-    <mergeCell ref="B289:E289"/>
-    <mergeCell ref="B290:E290"/>
-    <mergeCell ref="B291:E291"/>
-    <mergeCell ref="B292:E292"/>
-    <mergeCell ref="B458:E458"/>
-    <mergeCell ref="B466:E466"/>
-    <mergeCell ref="B467:E467"/>
-    <mergeCell ref="B468:E468"/>
-    <mergeCell ref="B426:E426"/>
-    <mergeCell ref="B438:E438"/>
-    <mergeCell ref="B439:E439"/>
-    <mergeCell ref="B453:E453"/>
-    <mergeCell ref="B454:E454"/>
-    <mergeCell ref="B455:E455"/>
-    <mergeCell ref="B456:E456"/>
-    <mergeCell ref="B457:E457"/>
-    <mergeCell ref="B442:E442"/>
-    <mergeCell ref="B450:E450"/>
-    <mergeCell ref="B451:E451"/>
-    <mergeCell ref="B387:E387"/>
-    <mergeCell ref="B389:E389"/>
-    <mergeCell ref="B390:E390"/>
-    <mergeCell ref="B392:E392"/>
-    <mergeCell ref="B403:E403"/>
-    <mergeCell ref="B404:E404"/>
-    <mergeCell ref="B406:E406"/>
-    <mergeCell ref="B409:E409"/>
-    <mergeCell ref="B377:E377"/>
-    <mergeCell ref="B378:E378"/>
-    <mergeCell ref="B379:E379"/>
-    <mergeCell ref="B388:E388"/>
-    <mergeCell ref="B395:E395"/>
-    <mergeCell ref="B400:E400"/>
-    <mergeCell ref="B402:E402"/>
-    <mergeCell ref="B393:E393"/>
-    <mergeCell ref="B396:E396"/>
-    <mergeCell ref="B398:E398"/>
-    <mergeCell ref="B399:E399"/>
-    <mergeCell ref="B401:E401"/>
-    <mergeCell ref="B386:E386"/>
-    <mergeCell ref="B505:E505"/>
-    <mergeCell ref="B480:E480"/>
-    <mergeCell ref="B469:E469"/>
-    <mergeCell ref="B481:E481"/>
-    <mergeCell ref="B490:E490"/>
-    <mergeCell ref="B491:E491"/>
-    <mergeCell ref="B492:E492"/>
-    <mergeCell ref="B493:E493"/>
-    <mergeCell ref="B494:E494"/>
-    <mergeCell ref="B498:E498"/>
-    <mergeCell ref="B499:E499"/>
-    <mergeCell ref="B500:E500"/>
-    <mergeCell ref="B501:E501"/>
-    <mergeCell ref="B502:E502"/>
-    <mergeCell ref="B503:E503"/>
-    <mergeCell ref="B504:E504"/>
-    <mergeCell ref="B482:E482"/>
-    <mergeCell ref="B495:E495"/>
-    <mergeCell ref="B511:E511"/>
-    <mergeCell ref="B512:E512"/>
-    <mergeCell ref="B513:E513"/>
-    <mergeCell ref="B514:E514"/>
-    <mergeCell ref="B515:E515"/>
-    <mergeCell ref="B535:E535"/>
-    <mergeCell ref="B537:E537"/>
-    <mergeCell ref="B555:E555"/>
-    <mergeCell ref="B560:E560"/>
-    <mergeCell ref="B548:E548"/>
-    <mergeCell ref="B549:E549"/>
-    <mergeCell ref="B546:E546"/>
-    <mergeCell ref="B547:E547"/>
-    <mergeCell ref="B533:E533"/>
-    <mergeCell ref="B534:E534"/>
-    <mergeCell ref="B536:E536"/>
-    <mergeCell ref="B538:E538"/>
-    <mergeCell ref="B539:E539"/>
-    <mergeCell ref="B540:E540"/>
-    <mergeCell ref="B541:E541"/>
-    <mergeCell ref="B543:E543"/>
-    <mergeCell ref="B544:E544"/>
-    <mergeCell ref="B526:E526"/>
-    <mergeCell ref="B527:E527"/>
-    <mergeCell ref="B569:E569"/>
-    <mergeCell ref="B570:E570"/>
-    <mergeCell ref="B571:E571"/>
-    <mergeCell ref="B572:E572"/>
-    <mergeCell ref="B573:E573"/>
-    <mergeCell ref="B576:E576"/>
-    <mergeCell ref="B578:E578"/>
-    <mergeCell ref="B591:E591"/>
-    <mergeCell ref="B592:E592"/>
-    <mergeCell ref="B580:E580"/>
-    <mergeCell ref="B589:E589"/>
-    <mergeCell ref="B594:E594"/>
-    <mergeCell ref="B627:E627"/>
-    <mergeCell ref="B647:E647"/>
-    <mergeCell ref="B661:E661"/>
-    <mergeCell ref="B662:E662"/>
-    <mergeCell ref="B663:E663"/>
-    <mergeCell ref="B664:E664"/>
-    <mergeCell ref="B665:E665"/>
-    <mergeCell ref="B666:E666"/>
-    <mergeCell ref="B633:E633"/>
-    <mergeCell ref="B634:E634"/>
-    <mergeCell ref="B635:E635"/>
-    <mergeCell ref="B611:E611"/>
-    <mergeCell ref="B628:E628"/>
-    <mergeCell ref="B629:E629"/>
-    <mergeCell ref="B630:E630"/>
-    <mergeCell ref="B631:E631"/>
-    <mergeCell ref="B632:E632"/>
-    <mergeCell ref="B621:E621"/>
-    <mergeCell ref="B622:E622"/>
-    <mergeCell ref="B623:E623"/>
-    <mergeCell ref="B624:E624"/>
-    <mergeCell ref="B625:E625"/>
-    <mergeCell ref="B600:E600"/>
-    <mergeCell ref="B677:E677"/>
-    <mergeCell ref="B678:E678"/>
-    <mergeCell ref="B680:E680"/>
-    <mergeCell ref="B681:E681"/>
-    <mergeCell ref="B682:E682"/>
-    <mergeCell ref="B683:E683"/>
-    <mergeCell ref="B684:E684"/>
-    <mergeCell ref="B685:E685"/>
-    <mergeCell ref="B686:E686"/>
-    <mergeCell ref="B703:E703"/>
-    <mergeCell ref="B706:E706"/>
-    <mergeCell ref="B707:E707"/>
-    <mergeCell ref="B708:E708"/>
-    <mergeCell ref="B709:E709"/>
-    <mergeCell ref="B710:E710"/>
-    <mergeCell ref="B711:E711"/>
-    <mergeCell ref="B712:E712"/>
-    <mergeCell ref="B693:E693"/>
-    <mergeCell ref="B722:E722"/>
-    <mergeCell ref="B723:E723"/>
-    <mergeCell ref="B724:E724"/>
-    <mergeCell ref="B725:E725"/>
-    <mergeCell ref="B704:E704"/>
-    <mergeCell ref="B726:E726"/>
-    <mergeCell ref="B713:E713"/>
-    <mergeCell ref="B714:E714"/>
-    <mergeCell ref="B715:E715"/>
-    <mergeCell ref="B716:E716"/>
-    <mergeCell ref="B717:E717"/>
-    <mergeCell ref="B718:E718"/>
-    <mergeCell ref="B719:E719"/>
-    <mergeCell ref="B720:E720"/>
-    <mergeCell ref="B721:E721"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="G56" r:id="rId1" display="106" xr:uid="{91711D96-DEE6-4487-B096-595B3971FA7B}"/>
@@ -55551,40 +55820,78 @@
       <c r="K226" s="22">
         <v>0</v>
       </c>
-      <c r="L226" s="15"/>
+      <c r="L226" s="15" t="s">
+        <v>301</v>
+      </c>
       <c r="M226" s="15"/>
     </row>
-    <row r="227" spans="1:13" ht="14.25">
+    <row r="227" spans="1:13">
       <c r="A227" s="14">
         <v>242</v>
       </c>
-      <c r="B227" s="42"/>
-      <c r="C227" s="61"/>
-      <c r="D227" s="61"/>
-      <c r="E227" s="61"/>
-      <c r="F227" s="62"/>
-      <c r="G227" s="61"/>
-      <c r="H227" s="62"/>
-      <c r="I227" s="61"/>
-      <c r="J227" s="15"/>
-      <c r="K227" s="22"/>
+      <c r="B227" s="42">
+        <v>46215</v>
+      </c>
+      <c r="C227" s="12" t="s">
+        <v>297</v>
+      </c>
+      <c r="D227" s="12" t="s">
+        <v>388</v>
+      </c>
+      <c r="E227" s="12" t="s">
+        <v>298</v>
+      </c>
+      <c r="F227" s="13">
+        <v>0.54861111111111116</v>
+      </c>
+      <c r="G227" s="12" t="s">
+        <v>342</v>
+      </c>
+      <c r="H227" s="13">
+        <v>0.60069444444444442</v>
+      </c>
+      <c r="I227" s="26"/>
+      <c r="J227" s="15" t="s">
+        <v>362</v>
+      </c>
+      <c r="K227" s="22">
+        <v>0</v>
+      </c>
       <c r="L227" s="15"/>
       <c r="M227" s="15"/>
     </row>
-    <row r="228" spans="1:13" ht="14.25">
+    <row r="228" spans="1:13">
       <c r="A228" s="14">
         <v>243</v>
       </c>
-      <c r="B228" s="42"/>
-      <c r="C228" s="61"/>
-      <c r="D228" s="61"/>
-      <c r="E228" s="61"/>
-      <c r="F228" s="62"/>
-      <c r="G228" s="61"/>
-      <c r="H228" s="62"/>
-      <c r="I228" s="61"/>
-      <c r="J228" s="15"/>
-      <c r="K228" s="22"/>
+      <c r="B228" s="42">
+        <v>46217</v>
+      </c>
+      <c r="C228" s="12" t="s">
+        <v>297</v>
+      </c>
+      <c r="D228" s="12" t="s">
+        <v>386</v>
+      </c>
+      <c r="E228" s="12" t="s">
+        <v>342</v>
+      </c>
+      <c r="F228" s="13">
+        <v>0.85763888888888884</v>
+      </c>
+      <c r="G228" s="12" t="s">
+        <v>298</v>
+      </c>
+      <c r="H228" s="13">
+        <v>0.91319444444444442</v>
+      </c>
+      <c r="I228" s="26"/>
+      <c r="J228" s="15" t="s">
+        <v>362</v>
+      </c>
+      <c r="K228" s="22">
+        <v>0</v>
+      </c>
       <c r="L228" s="15"/>
       <c r="M228" s="15"/>
     </row>
@@ -56185,7 +56492,7 @@
     </row>
     <row r="274" spans="10:11">
       <c r="J274" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="K274" s="11">
         <f>SUM(テーブル4[料金])</f>
@@ -56194,11 +56501,11 @@
     </row>
     <row r="275" spans="10:11">
       <c r="J275" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="K275">
         <f>COUNTA(テーブル4[料金])*5</f>
-        <v>1105</v>
+        <v>1115</v>
       </c>
     </row>
     <row r="276" spans="10:11">
@@ -56207,16 +56514,16 @@
       </c>
       <c r="K276">
         <f>COUNTA(テーブル4[料金])</f>
-        <v>221</v>
+        <v>223</v>
       </c>
     </row>
     <row r="277" spans="10:11">
       <c r="J277" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="K277" s="41">
         <f>K274/K275</f>
-        <v>1233.9583710407239</v>
+        <v>1222.8914798206279</v>
       </c>
     </row>
     <row r="289" spans="1:8">
@@ -56294,7 +56601,7 @@
         <v>0.43402777777777779</v>
       </c>
       <c r="H291" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
     </row>
     <row r="292" spans="1:8">
@@ -56346,7 +56653,7 @@
         <v>0.57291666666666663</v>
       </c>
       <c r="H293" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
     </row>
     <row r="294" spans="1:8">
@@ -56450,7 +56757,7 @@
         <v>0.91666666666666663</v>
       </c>
       <c r="H297" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
     </row>
     <row r="300" spans="1:8">
@@ -56684,7 +56991,7 @@
         <v>0.375</v>
       </c>
       <c r="H309" s="51" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="I309" s="52"/>
     </row>
@@ -56738,7 +57045,7 @@
         <v>0.54513888888888884</v>
       </c>
       <c r="H311" s="49" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="I311" s="52"/>
     </row>
@@ -56873,7 +57180,7 @@
         <v>0.78472222222222221</v>
       </c>
       <c r="H316" s="54" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="I316" s="56"/>
     </row>

</xml_diff>

<commit_message>
Fix flight count aggregation and update LSP management data
</commit_message>
<xml_diff>
--- a/data/20251229_LSP管理.xlsx
+++ b/data/20251229_LSP管理.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hiraizumitatsuya/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B1793B22-65D6-4830-907D-B3B2E1BB56D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{3B253F34-1BD6-465A-B220-1B923CA0921D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="33600" windowHeight="20500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2992" uniqueCount="397">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3019" uniqueCount="403">
   <si>
     <t>日付</t>
   </si>
@@ -1219,6 +1219,24 @@
     <t>JAL481</t>
   </si>
   <si>
+    <t>JAL503</t>
+  </si>
+  <si>
+    <t>札幌（新千歳）</t>
+  </si>
+  <si>
+    <t>JAL524</t>
+  </si>
+  <si>
+    <t>JAL153</t>
+  </si>
+  <si>
+    <t>三沢</t>
+  </si>
+  <si>
+    <t>JAL158</t>
+  </si>
+  <si>
     <t>総額</t>
   </si>
   <si>
@@ -2394,7 +2412,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0" formatCode="#,##0">
-                  <c:v>128359</c:v>
+                  <c:v>129223</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>60787</c:v>
@@ -2406,7 +2424,7 @@
                   <c:v>2000</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>6884</c:v>
+                  <c:v>6914</c:v>
                 </c:pt>
                 <c:pt idx="5">
                   <c:v>144</c:v>
@@ -15045,7 +15063,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2A57836D-5153-486D-8B76-48FAFDDE1EA1}">
-  <dimension ref="A1:O733"/>
+  <dimension ref="A1:O735"/>
   <sheetFormatPr defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="13.7109375" customWidth="1"/>
@@ -15441,7 +15459,7 @@
       </c>
       <c r="O12" s="11">
         <f>SUMIFS(H2:H29999, B2:B29999, "*JL*")+SUMIFS(H11:H29999, B11:B29999, "*NU*")</f>
-        <v>128359</v>
+        <v>129223</v>
       </c>
     </row>
     <row r="13" spans="1:15">
@@ -15613,7 +15631,7 @@
       </c>
       <c r="O16">
         <f>SUMIFS(H11:H29999, B11:B29999, "*ＷＥＬＬＮＥＳＳ*")</f>
-        <v>6884</v>
+        <v>6914</v>
       </c>
     </row>
     <row r="17" spans="1:15">
@@ -15855,7 +15873,7 @@
       <c r="N21" s="31"/>
       <c r="O21">
         <f>SUM(O12:O18)</f>
-        <v>168174</v>
+        <v>169068</v>
       </c>
     </row>
     <row r="22" spans="1:15">
@@ -43261,37 +43279,43 @@
       <c r="A729" s="27">
         <v>46199</v>
       </c>
-      <c r="B729" s="76" t="s">
-        <v>49</v>
-      </c>
-      <c r="C729" s="76"/>
-      <c r="D729" s="76"/>
-      <c r="E729" s="77"/>
+      <c r="B729" s="1" t="s">
+        <v>236</v>
+      </c>
+      <c r="C729" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="D729" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="E729" s="1" t="s">
+        <v>50</v>
+      </c>
       <c r="F729" s="74">
-        <v>0</v>
-      </c>
-      <c r="G729" s="74">
+        <v>354</v>
+      </c>
+      <c r="G729" s="28">
+        <v>510</v>
+      </c>
+      <c r="H729" s="74">
+        <v>864</v>
+      </c>
+      <c r="I729" s="4">
+        <v>82450</v>
+      </c>
+      <c r="J729" s="4">
+        <v>1108</v>
+      </c>
+      <c r="K729" s="74">
         <v>1</v>
-      </c>
-      <c r="H729" s="74">
-        <v>1</v>
-      </c>
-      <c r="I729" s="4">
-        <v>81587</v>
-      </c>
-      <c r="J729" s="74">
-        <v>0</v>
-      </c>
-      <c r="K729" s="74">
-        <v>0</v>
       </c>
       <c r="L729" s="74">
         <f t="shared" si="104"/>
-        <v>85476</v>
+        <v>86584</v>
       </c>
       <c r="M729" s="74">
         <f t="shared" si="105"/>
-        <v>133</v>
+        <v>134</v>
       </c>
     </row>
     <row r="730" spans="1:13">
@@ -43299,7 +43323,7 @@
         <v>46199</v>
       </c>
       <c r="B730" s="76" t="s">
-        <v>33</v>
+        <v>49</v>
       </c>
       <c r="C730" s="76"/>
       <c r="D730" s="76"/>
@@ -43308,13 +43332,13 @@
         <v>0</v>
       </c>
       <c r="G730" s="74">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="H730" s="74">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="I730" s="4">
-        <v>81598</v>
+        <v>82451</v>
       </c>
       <c r="J730" s="74">
         <v>0</v>
@@ -43324,11 +43348,11 @@
       </c>
       <c r="L730" s="74">
         <f t="shared" si="104"/>
-        <v>85476</v>
+        <v>86584</v>
       </c>
       <c r="M730" s="74">
         <f t="shared" si="105"/>
-        <v>133</v>
+        <v>134</v>
       </c>
     </row>
     <row r="731" spans="1:13">
@@ -43336,7 +43360,7 @@
         <v>46199</v>
       </c>
       <c r="B731" s="76" t="s">
-        <v>49</v>
+        <v>33</v>
       </c>
       <c r="C731" s="76"/>
       <c r="D731" s="76"/>
@@ -43345,13 +43369,13 @@
         <v>0</v>
       </c>
       <c r="G731" s="74">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="H731" s="74">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="I731" s="4">
-        <v>81599</v>
+        <v>82462</v>
       </c>
       <c r="J731" s="74">
         <v>0</v>
@@ -43361,11 +43385,11 @@
       </c>
       <c r="L731" s="74">
         <f t="shared" si="104"/>
-        <v>85476</v>
+        <v>86584</v>
       </c>
       <c r="M731" s="74">
         <f t="shared" si="105"/>
-        <v>133</v>
+        <v>134</v>
       </c>
     </row>
     <row r="732" spans="1:13">
@@ -43388,7 +43412,7 @@
         <v>1</v>
       </c>
       <c r="I732" s="4">
-        <v>81600</v>
+        <v>82463</v>
       </c>
       <c r="J732" s="74">
         <v>0</v>
@@ -43398,56 +43422,131 @@
       </c>
       <c r="L732" s="74">
         <f t="shared" si="104"/>
-        <v>85476</v>
+        <v>86584</v>
       </c>
       <c r="M732" s="74">
         <f t="shared" si="105"/>
-        <v>133</v>
+        <v>134</v>
       </c>
     </row>
     <row r="733" spans="1:13">
-      <c r="A733" s="29">
-        <v>46200</v>
-      </c>
-      <c r="B733" s="78" t="s">
-        <v>33</v>
-      </c>
-      <c r="C733" s="78"/>
-      <c r="D733" s="78"/>
-      <c r="E733" s="79"/>
-      <c r="F733" s="75">
-        <v>0</v>
-      </c>
-      <c r="G733" s="75">
-        <v>9</v>
-      </c>
-      <c r="H733" s="75">
-        <v>9</v>
-      </c>
-      <c r="I733" s="30">
-        <v>81609</v>
-      </c>
-      <c r="J733" s="75">
-        <v>0</v>
-      </c>
-      <c r="K733" s="75">
+      <c r="A733" s="27">
+        <v>46199</v>
+      </c>
+      <c r="B733" s="76" t="s">
+        <v>49</v>
+      </c>
+      <c r="C733" s="76"/>
+      <c r="D733" s="76"/>
+      <c r="E733" s="77"/>
+      <c r="F733" s="74">
+        <v>0</v>
+      </c>
+      <c r="G733" s="74">
+        <v>1</v>
+      </c>
+      <c r="H733" s="74">
+        <v>1</v>
+      </c>
+      <c r="I733" s="4">
+        <v>82464</v>
+      </c>
+      <c r="J733" s="74">
+        <v>0</v>
+      </c>
+      <c r="K733" s="74">
         <v>0</v>
       </c>
       <c r="L733" s="74">
         <f t="shared" si="104"/>
-        <v>85476</v>
+        <v>86584</v>
       </c>
       <c r="M733" s="74">
         <f t="shared" si="105"/>
-        <v>133</v>
+        <v>134</v>
+      </c>
+    </row>
+    <row r="734" spans="1:13">
+      <c r="A734" s="27">
+        <v>46200</v>
+      </c>
+      <c r="B734" s="76" t="s">
+        <v>33</v>
+      </c>
+      <c r="C734" s="76"/>
+      <c r="D734" s="76"/>
+      <c r="E734" s="77"/>
+      <c r="F734" s="74">
+        <v>0</v>
+      </c>
+      <c r="G734" s="74">
+        <v>9</v>
+      </c>
+      <c r="H734" s="74">
+        <v>9</v>
+      </c>
+      <c r="I734" s="4">
+        <v>82473</v>
+      </c>
+      <c r="J734" s="74">
+        <v>0</v>
+      </c>
+      <c r="K734" s="74">
+        <v>0</v>
+      </c>
+      <c r="L734" s="74">
+        <f t="shared" ref="L734:L735" si="106">J734+L733</f>
+        <v>86584</v>
+      </c>
+      <c r="M734" s="74">
+        <f t="shared" ref="M734:M735" si="107">K734+M733</f>
+        <v>134</v>
+      </c>
+    </row>
+    <row r="735" spans="1:13">
+      <c r="A735" s="29">
+        <v>46201</v>
+      </c>
+      <c r="B735" s="78" t="s">
+        <v>33</v>
+      </c>
+      <c r="C735" s="78"/>
+      <c r="D735" s="78"/>
+      <c r="E735" s="79"/>
+      <c r="F735" s="75">
+        <v>0</v>
+      </c>
+      <c r="G735" s="75">
+        <v>30</v>
+      </c>
+      <c r="H735" s="75">
+        <v>30</v>
+      </c>
+      <c r="I735" s="30">
+        <v>82503</v>
+      </c>
+      <c r="J735" s="75">
+        <v>0</v>
+      </c>
+      <c r="K735" s="75">
+        <v>0</v>
+      </c>
+      <c r="L735" s="74">
+        <f t="shared" si="106"/>
+        <v>86584</v>
+      </c>
+      <c r="M735" s="74">
+        <f t="shared" si="107"/>
+        <v>134</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:O523" xr:uid="{2A57836D-5153-486D-8B76-48FAFDDE1EA1}"/>
-  <mergeCells count="506">
+  <mergeCells count="507">
+    <mergeCell ref="B734:E734"/>
+    <mergeCell ref="B735:E735"/>
     <mergeCell ref="B727:E727"/>
     <mergeCell ref="B728:E728"/>
-    <mergeCell ref="B729:E729"/>
     <mergeCell ref="B730:E730"/>
     <mergeCell ref="B731:E731"/>
     <mergeCell ref="B732:E732"/>
@@ -44147,9 +44246,10 @@
     <hyperlink ref="G700" r:id="rId192" display="863" xr:uid="{95F5C9F2-6065-40BF-AD9E-E67580350D2F}"/>
     <hyperlink ref="G702" r:id="rId193" display="560" xr:uid="{579C9D04-A680-4706-887F-9A090C67F828}"/>
     <hyperlink ref="G705" r:id="rId194" display="560" xr:uid="{23497521-CF0C-4006-A8C3-37035833FC60}"/>
+    <hyperlink ref="G729" r:id="rId195" display="510" xr:uid="{47E037CC-A9E7-41D0-9CD9-CE09618E527A}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId195"/>
+  <drawing r:id="rId196"/>
 </worksheet>
 </file>
 
@@ -55895,72 +55995,148 @@
       <c r="L228" s="15"/>
       <c r="M228" s="15"/>
     </row>
-    <row r="229" spans="1:13" ht="14.25">
+    <row r="229" spans="1:13">
       <c r="A229" s="14">
         <v>244</v>
       </c>
-      <c r="B229" s="42"/>
-      <c r="C229" s="61"/>
-      <c r="D229" s="61"/>
-      <c r="E229" s="61"/>
-      <c r="F229" s="62"/>
-      <c r="G229" s="61"/>
-      <c r="H229" s="62"/>
-      <c r="I229" s="61"/>
-      <c r="J229" s="15"/>
-      <c r="K229" s="22"/>
+      <c r="B229" s="42">
+        <v>46204</v>
+      </c>
+      <c r="C229" s="12" t="s">
+        <v>297</v>
+      </c>
+      <c r="D229" s="12" t="s">
+        <v>389</v>
+      </c>
+      <c r="E229" s="12" t="s">
+        <v>298</v>
+      </c>
+      <c r="F229" s="13">
+        <v>0.30208333333333331</v>
+      </c>
+      <c r="G229" s="12" t="s">
+        <v>390</v>
+      </c>
+      <c r="H229" s="13">
+        <v>0.36805555555555558</v>
+      </c>
+      <c r="I229" s="26"/>
+      <c r="J229" s="15" t="s">
+        <v>362</v>
+      </c>
+      <c r="K229" s="22">
+        <v>0</v>
+      </c>
       <c r="L229" s="15"/>
       <c r="M229" s="15"/>
     </row>
-    <row r="230" spans="1:13" ht="14.25">
+    <row r="230" spans="1:13">
       <c r="A230" s="14">
         <v>245</v>
       </c>
-      <c r="B230" s="42"/>
-      <c r="C230" s="61"/>
-      <c r="D230" s="61"/>
-      <c r="E230" s="61"/>
-      <c r="F230" s="62"/>
-      <c r="G230" s="61"/>
-      <c r="H230" s="62"/>
-      <c r="I230" s="61"/>
-      <c r="J230" s="15"/>
-      <c r="K230" s="22"/>
+      <c r="B230" s="42">
+        <v>46204</v>
+      </c>
+      <c r="C230" s="12" t="s">
+        <v>297</v>
+      </c>
+      <c r="D230" s="12" t="s">
+        <v>391</v>
+      </c>
+      <c r="E230" s="12" t="s">
+        <v>390</v>
+      </c>
+      <c r="F230" s="13">
+        <v>0.80208333333333337</v>
+      </c>
+      <c r="G230" s="12" t="s">
+        <v>298</v>
+      </c>
+      <c r="H230" s="13">
+        <v>0.87152777777777779</v>
+      </c>
+      <c r="I230" s="26"/>
+      <c r="J230" s="15" t="s">
+        <v>362</v>
+      </c>
+      <c r="K230" s="22">
+        <v>0</v>
+      </c>
       <c r="L230" s="15"/>
       <c r="M230" s="15"/>
     </row>
-    <row r="231" spans="1:13" ht="14.25">
+    <row r="231" spans="1:13">
       <c r="A231" s="14">
         <v>246</v>
       </c>
-      <c r="B231" s="42"/>
-      <c r="C231" s="61"/>
-      <c r="D231" s="61"/>
-      <c r="E231" s="61"/>
-      <c r="F231" s="62"/>
-      <c r="G231" s="61"/>
-      <c r="H231" s="62"/>
-      <c r="I231" s="61"/>
-      <c r="J231" s="15"/>
-      <c r="K231" s="22"/>
-      <c r="L231" s="15"/>
+      <c r="B231" s="42">
+        <v>46177</v>
+      </c>
+      <c r="C231" s="12" t="s">
+        <v>297</v>
+      </c>
+      <c r="D231" s="12" t="s">
+        <v>392</v>
+      </c>
+      <c r="E231" s="12" t="s">
+        <v>298</v>
+      </c>
+      <c r="F231" s="13">
+        <v>0.30208333333333331</v>
+      </c>
+      <c r="G231" s="12" t="s">
+        <v>393</v>
+      </c>
+      <c r="H231" s="13">
+        <v>0.36805555555555558</v>
+      </c>
+      <c r="I231" s="26"/>
+      <c r="J231" s="15" t="s">
+        <v>362</v>
+      </c>
+      <c r="K231" s="22">
+        <v>0</v>
+      </c>
+      <c r="L231" s="15" t="s">
+        <v>301</v>
+      </c>
       <c r="M231" s="15"/>
     </row>
-    <row r="232" spans="1:13" ht="14.25">
+    <row r="232" spans="1:13">
       <c r="A232" s="14">
         <v>247</v>
       </c>
-      <c r="B232" s="42"/>
-      <c r="C232" s="61"/>
-      <c r="D232" s="61"/>
-      <c r="E232" s="61"/>
-      <c r="F232" s="62"/>
-      <c r="G232" s="61"/>
-      <c r="H232" s="62"/>
-      <c r="I232" s="61"/>
-      <c r="J232" s="15"/>
-      <c r="K232" s="22"/>
-      <c r="L232" s="15"/>
+      <c r="B232" s="42">
+        <v>46177</v>
+      </c>
+      <c r="C232" s="12" t="s">
+        <v>297</v>
+      </c>
+      <c r="D232" s="12" t="s">
+        <v>394</v>
+      </c>
+      <c r="E232" s="12" t="s">
+        <v>393</v>
+      </c>
+      <c r="F232" s="13">
+        <v>0.80208333333333337</v>
+      </c>
+      <c r="G232" s="12" t="s">
+        <v>298</v>
+      </c>
+      <c r="H232" s="13">
+        <v>0.87152777777777779</v>
+      </c>
+      <c r="I232" s="26"/>
+      <c r="J232" s="15" t="s">
+        <v>362</v>
+      </c>
+      <c r="K232" s="22">
+        <v>0</v>
+      </c>
+      <c r="L232" s="15" t="s">
+        <v>301</v>
+      </c>
       <c r="M232" s="15"/>
     </row>
     <row r="233" spans="1:13" ht="14.25">
@@ -56492,7 +56668,7 @@
     </row>
     <row r="274" spans="10:11">
       <c r="J274" t="s">
-        <v>389</v>
+        <v>395</v>
       </c>
       <c r="K274" s="11">
         <f>SUM(テーブル4[料金])</f>
@@ -56501,11 +56677,11 @@
     </row>
     <row r="275" spans="10:11">
       <c r="J275" t="s">
-        <v>390</v>
+        <v>396</v>
       </c>
       <c r="K275">
         <f>COUNTA(テーブル4[料金])*5</f>
-        <v>1115</v>
+        <v>1135</v>
       </c>
     </row>
     <row r="276" spans="10:11">
@@ -56514,16 +56690,16 @@
       </c>
       <c r="K276">
         <f>COUNTA(テーブル4[料金])</f>
-        <v>223</v>
+        <v>227</v>
       </c>
     </row>
     <row r="277" spans="10:11">
       <c r="J277" t="s">
-        <v>391</v>
+        <v>397</v>
       </c>
       <c r="K277" s="41">
         <f>K274/K275</f>
-        <v>1222.8914798206279</v>
+        <v>1201.3427312775329</v>
       </c>
     </row>
     <row r="289" spans="1:8">
@@ -56601,7 +56777,7 @@
         <v>0.43402777777777779</v>
       </c>
       <c r="H291" t="s">
-        <v>392</v>
+        <v>398</v>
       </c>
     </row>
     <row r="292" spans="1:8">
@@ -56653,7 +56829,7 @@
         <v>0.57291666666666663</v>
       </c>
       <c r="H293" t="s">
-        <v>393</v>
+        <v>399</v>
       </c>
     </row>
     <row r="294" spans="1:8">
@@ -56757,7 +56933,7 @@
         <v>0.91666666666666663</v>
       </c>
       <c r="H297" t="s">
-        <v>394</v>
+        <v>400</v>
       </c>
     </row>
     <row r="300" spans="1:8">
@@ -56991,7 +57167,7 @@
         <v>0.375</v>
       </c>
       <c r="H309" s="51" t="s">
-        <v>395</v>
+        <v>401</v>
       </c>
       <c r="I309" s="52"/>
     </row>
@@ -57045,7 +57221,7 @@
         <v>0.54513888888888884</v>
       </c>
       <c r="H311" s="49" t="s">
-        <v>396</v>
+        <v>402</v>
       </c>
       <c r="I311" s="52"/>
     </row>
@@ -57180,7 +57356,7 @@
         <v>0.78472222222222221</v>
       </c>
       <c r="H316" s="54" t="s">
-        <v>394</v>
+        <v>400</v>
       </c>
       <c r="I316" s="56"/>
     </row>

</xml_diff>